<commit_message>
chore: sinkronisasi branding & palet warna — prefix AAJ, API URL, docker, palet #2596BE
- Backlog/GitHub Projects/QA Test Plan/issue template: prefix story BW- (BukuWarung) → AAJ- (Appsheet Accounting Journal); regenerate qa-test-cases CSV/XLSX agar pemetaan AC/sprint tetap konsisten
- API base URL api.bukuwarung.com → api.appsheetaccountingjournal.com (API - Accounting.md, openapi.yaml, TRD VITE_API_URL)
- Docker image bukuwarung-akuntansi → appsheet-accounting-journal (TRD)
- Baru: Color Palette - Accounting.md — referensi palet lengkap light + dark, brand #2596BE, peta token ke semua modul

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/qa-test-cases.xlsx
+++ b/qa-test-cases.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>BW-001</t>
+          <t>AAJ-001</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>BW-001</t>
+          <t>AAJ-001</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>BW-001</t>
+          <t>AAJ-001</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>BW-002</t>
+          <t>AAJ-002</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>BW-001</t>
+          <t>AAJ-001</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>BW-001</t>
+          <t>AAJ-001</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>BW-002</t>
+          <t>AAJ-002</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>BW-003</t>
+          <t>AAJ-003</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>BW-003</t>
+          <t>AAJ-003</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>BW-003</t>
+          <t>AAJ-003</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>BW-003</t>
+          <t>AAJ-003</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>BW-004</t>
+          <t>AAJ-004</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>BW-005</t>
+          <t>AAJ-005</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>BW-005</t>
+          <t>AAJ-005</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>BW-033</t>
+          <t>AAJ-033</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>BW-033</t>
+          <t>AAJ-033</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>BW-006</t>
+          <t>AAJ-006</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>BW-007</t>
+          <t>AAJ-007</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>BW-007</t>
+          <t>AAJ-007</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>BW-007</t>
+          <t>AAJ-007</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>BW-008</t>
+          <t>AAJ-008</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>BW-008</t>
+          <t>AAJ-008</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>BW-008</t>
+          <t>AAJ-008</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>BW-008</t>
+          <t>AAJ-008</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>BW-008</t>
+          <t>AAJ-008</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>BW-008</t>
+          <t>AAJ-008</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>BW-009</t>
+          <t>AAJ-009</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>BW-009</t>
+          <t>AAJ-009</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>BW-009</t>
+          <t>AAJ-009</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>BW-009</t>
+          <t>AAJ-009</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>BW-013</t>
+          <t>AAJ-013</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>BW-013</t>
+          <t>AAJ-013</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>BW-010</t>
+          <t>AAJ-010</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>BW-010</t>
+          <t>AAJ-010</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>BW-010</t>
+          <t>AAJ-010</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4123,7 +4123,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>BW-010</t>
+          <t>AAJ-010</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>BW-010</t>
+          <t>AAJ-010</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>BW-010</t>
+          <t>AAJ-010</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>BW-011</t>
+          <t>AAJ-011</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>BW-011</t>
+          <t>AAJ-011</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>BW-011</t>
+          <t>AAJ-011</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>BW-011</t>
+          <t>AAJ-011</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>BW-011</t>
+          <t>AAJ-011</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>BW-011</t>
+          <t>AAJ-011</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>BW-027</t>
+          <t>AAJ-027</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>BW-027</t>
+          <t>AAJ-027</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>BW-012</t>
+          <t>AAJ-012</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>BW-012</t>
+          <t>AAJ-012</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>BW-012</t>
+          <t>AAJ-012</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>BW-012</t>
+          <t>AAJ-012</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>BW-012</t>
+          <t>AAJ-012</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>BW-012</t>
+          <t>AAJ-012</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>BW-019</t>
+          <t>AAJ-019</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>BW-014</t>
+          <t>AAJ-014</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>BW-014</t>
+          <t>AAJ-014</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
@@ -5563,7 +5563,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>BW-014</t>
+          <t>AAJ-014</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>BW-015</t>
+          <t>AAJ-015</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -5707,7 +5707,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>BW-015</t>
+          <t>AAJ-015</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>BW-015</t>
+          <t>AAJ-015</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>BW-015</t>
+          <t>AAJ-015</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>BW-014</t>
+          <t>AAJ-014</t>
         </is>
       </c>
       <c r="H76" s="5" t="inlineStr">
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>BW-014</t>
+          <t>AAJ-014</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>BW-016</t>
+          <t>AAJ-016</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>BW-016</t>
+          <t>AAJ-016</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>BW-016</t>
+          <t>AAJ-016</t>
         </is>
       </c>
       <c r="H80" s="5" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>BW-016</t>
+          <t>AAJ-016</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>BW-017</t>
+          <t>AAJ-017</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>BW-017</t>
+          <t>AAJ-017</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -6499,7 +6499,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>BW-017</t>
+          <t>AAJ-017</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>BW-018</t>
+          <t>AAJ-018</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -6643,7 +6643,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>BW-018</t>
+          <t>AAJ-018</t>
         </is>
       </c>
       <c r="H86" s="5" t="inlineStr">
@@ -6715,7 +6715,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>BW-018</t>
+          <t>AAJ-018</t>
         </is>
       </c>
       <c r="H87" s="5" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>BW-031</t>
+          <t>AAJ-031</t>
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr">
@@ -6859,7 +6859,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>BW-020</t>
+          <t>AAJ-020</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -6931,7 +6931,7 @@
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>BW-020</t>
+          <t>AAJ-020</t>
         </is>
       </c>
       <c r="H90" s="5" t="inlineStr">
@@ -7003,7 +7003,7 @@
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>BW-020</t>
+          <t>AAJ-020</t>
         </is>
       </c>
       <c r="H91" s="5" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>BW-020</t>
+          <t>AAJ-020</t>
         </is>
       </c>
       <c r="H92" s="5" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>BW-021</t>
+          <t>AAJ-021</t>
         </is>
       </c>
       <c r="H93" s="5" t="inlineStr">
@@ -7219,7 +7219,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>BW-020</t>
+          <t>AAJ-020</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>BW-022</t>
+          <t>AAJ-022</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>BW-022</t>
+          <t>AAJ-022</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -7499,7 +7499,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>BW-022</t>
+          <t>AAJ-022</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -7571,7 +7571,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>BW-022</t>
+          <t>AAJ-022</t>
         </is>
       </c>
       <c r="H99" s="5" t="inlineStr">
@@ -7643,7 +7643,7 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>BW-022</t>
+          <t>AAJ-022</t>
         </is>
       </c>
       <c r="H100" s="5" t="inlineStr">
@@ -7715,7 +7715,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>BW-023</t>
+          <t>AAJ-023</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -7787,7 +7787,7 @@
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>BW-023</t>
+          <t>AAJ-023</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr">
@@ -7859,7 +7859,7 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>BW-023</t>
+          <t>AAJ-023</t>
         </is>
       </c>
       <c r="H103" s="5" t="inlineStr">
@@ -7931,7 +7931,7 @@
       </c>
       <c r="G104" s="5" t="inlineStr">
         <is>
-          <t>BW-023</t>
+          <t>AAJ-023</t>
         </is>
       </c>
       <c r="H104" s="5" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>BW-024</t>
+          <t>AAJ-024</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -8075,7 +8075,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>BW-024</t>
+          <t>AAJ-024</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
-          <t>BW-024</t>
+          <t>AAJ-024</t>
         </is>
       </c>
       <c r="H107" s="5" t="inlineStr">
@@ -8219,7 +8219,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>BW-024</t>
+          <t>AAJ-024</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>BW-024</t>
+          <t>AAJ-024</t>
         </is>
       </c>
       <c r="H109" s="5" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="G110" s="5" t="inlineStr">
         <is>
-          <t>BW-024</t>
+          <t>AAJ-024</t>
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>BW-025</t>
+          <t>AAJ-025</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -8507,7 +8507,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>BW-025</t>
+          <t>AAJ-025</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>BW-025</t>
+          <t>AAJ-025</t>
         </is>
       </c>
       <c r="H113" s="5" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="G114" s="5" t="inlineStr">
         <is>
-          <t>BW-025</t>
+          <t>AAJ-025</t>
         </is>
       </c>
       <c r="H114" s="5" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>BW-026</t>
+          <t>AAJ-026</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>BW-026</t>
+          <t>AAJ-026</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
-          <t>BW-026</t>
+          <t>AAJ-026</t>
         </is>
       </c>
       <c r="H117" s="5" t="inlineStr">
@@ -8939,7 +8939,7 @@
       </c>
       <c r="G118" s="5" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H118" s="5" t="inlineStr">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
@@ -9083,7 +9083,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -9155,7 +9155,7 @@
       </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H121" s="5" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr">
@@ -9299,7 +9299,7 @@
       </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H123" s="5" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H124" s="5" t="inlineStr">
@@ -9443,7 +9443,7 @@
       </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
-          <t>BW-029</t>
+          <t>AAJ-029</t>
         </is>
       </c>
       <c r="H125" s="5" t="inlineStr">
@@ -9515,7 +9515,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>BW-030</t>
+          <t>AAJ-030</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>BW-030</t>
+          <t>AAJ-030</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="G128" s="5" t="inlineStr">
         <is>
-          <t>BW-030</t>
+          <t>AAJ-030</t>
         </is>
       </c>
       <c r="H128" s="5" t="inlineStr">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
-          <t>BW-030</t>
+          <t>AAJ-030</t>
         </is>
       </c>
       <c r="H129" s="5" t="inlineStr">
@@ -9803,7 +9803,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>BW-032</t>
+          <t>AAJ-032</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
-          <t>BW-032</t>
+          <t>AAJ-032</t>
         </is>
       </c>
       <c r="H131" s="5" t="inlineStr">
@@ -9947,7 +9947,7 @@
       </c>
       <c r="G132" s="5" t="inlineStr">
         <is>
-          <t>BW-032</t>
+          <t>AAJ-032</t>
         </is>
       </c>
       <c r="H132" s="5" t="inlineStr">
@@ -10019,7 +10019,7 @@
       </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
-          <t>BW-034</t>
+          <t>AAJ-034</t>
         </is>
       </c>
       <c r="H133" s="5" t="inlineStr">
@@ -10091,7 +10091,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>BW-034</t>
+          <t>AAJ-034</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -10163,7 +10163,7 @@
       </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
-          <t>BW-034</t>
+          <t>AAJ-034</t>
         </is>
       </c>
       <c r="H135" s="5" t="inlineStr">
@@ -10955,7 +10955,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>BW-028</t>
+          <t>AAJ-028</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr">
@@ -11027,7 +11027,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>BW-028</t>
+          <t>AAJ-028</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
@@ -11099,7 +11099,7 @@
       </c>
       <c r="G150" s="5" t="inlineStr">
         <is>
-          <t>BW-028</t>
+          <t>AAJ-028</t>
         </is>
       </c>
       <c r="H150" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(qa): generator hasil test + konverter payload TestRail, CF status, pertahankan status
- generate-qa-test-cases.py: regenerasi mempertahankan Status yang sudah
  diisi QA (baca dari qa-test-cases.xlsx, fallback tracker CSV) — hanya
  case baru/kosong yang di-set 'Not Run'
- generate-qa-test-cases.py: conditional formatting kolom Status di kedua
  XLSX (Passed hijau, Fail/Failed merah, Not Run abu-abu, Blocked/Retest
  amber, Skipped biru-abu) — warna ikut nilai sel saat diedit di Excel
- convert-results-to-testrail.py (baru): qa-test-results-testrail.csv →
  JSON payload add_results_for_cases (status_id 1/2/4/5/6, Not Run
  dilewati, case_id numerik atau via --mapping) + contoh curl
- Output QA di-regenerasi: tracker CSV & kedua XLSX dengan tanggal run
  hari ini dan conditional formatting

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/qa-test-cases.xlsx
+++ b/qa-test-cases.xlsx
@@ -110,6 +110,63 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001F4E78"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DDEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -610,7 +667,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -682,7 +739,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -754,7 +811,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -826,7 +883,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -898,7 +955,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -970,7 +1027,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1042,7 +1099,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1114,7 +1171,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1186,7 +1243,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1258,7 +1315,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1330,7 +1387,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1402,7 +1459,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1474,7 +1531,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1546,7 +1603,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1618,7 +1675,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -1690,7 +1747,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1762,7 +1819,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -1834,7 +1891,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -1906,7 +1963,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1978,7 +2035,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -2050,7 +2107,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2122,7 +2179,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -2194,7 +2251,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2266,7 +2323,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2338,7 +2395,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2410,7 +2467,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -2482,7 +2539,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -2554,7 +2611,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2626,7 +2683,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -2698,7 +2755,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -2770,7 +2827,7 @@
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -2842,7 +2899,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -2914,7 +2971,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -2986,7 +3043,7 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -3058,7 +3115,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3130,7 +3187,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3202,7 +3259,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3274,7 +3331,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -3346,7 +3403,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -3418,7 +3475,7 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
@@ -3490,7 +3547,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3562,7 +3619,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3634,7 +3691,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
@@ -3706,7 +3763,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
@@ -3778,7 +3835,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -3850,7 +3907,7 @@
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
@@ -3922,7 +3979,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -3994,7 +4051,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4066,7 +4123,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4138,7 +4195,7 @@
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
@@ -4210,7 +4267,7 @@
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
@@ -4282,7 +4339,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
@@ -4354,7 +4411,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -4426,7 +4483,7 @@
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
@@ -4498,7 +4555,7 @@
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
@@ -4570,7 +4627,7 @@
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
@@ -4642,7 +4699,7 @@
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
@@ -4714,7 +4771,7 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
@@ -4786,7 +4843,7 @@
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
@@ -4858,7 +4915,7 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
@@ -4930,7 +4987,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5002,7 +5059,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -5074,7 +5131,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -5146,7 +5203,7 @@
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
@@ -5218,7 +5275,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -5290,7 +5347,7 @@
       </c>
       <c r="J67" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K67" s="5" t="inlineStr">
@@ -5362,7 +5419,7 @@
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
@@ -5434,7 +5491,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
@@ -5506,7 +5563,7 @@
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
@@ -5578,7 +5635,7 @@
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
@@ -5650,7 +5707,7 @@
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K72" s="5" t="inlineStr">
@@ -5722,7 +5779,7 @@
       </c>
       <c r="J73" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K73" s="5" t="inlineStr">
@@ -5794,7 +5851,7 @@
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K74" s="5" t="inlineStr">
@@ -5866,7 +5923,7 @@
       </c>
       <c r="J75" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K75" s="5" t="inlineStr">
@@ -5938,7 +5995,7 @@
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K76" s="5" t="inlineStr">
@@ -6010,7 +6067,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -6082,7 +6139,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
@@ -6154,7 +6211,7 @@
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
@@ -6226,7 +6283,7 @@
       </c>
       <c r="J80" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K80" s="5" t="inlineStr">
@@ -6298,7 +6355,7 @@
       </c>
       <c r="J81" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K81" s="5" t="inlineStr">
@@ -6370,7 +6427,7 @@
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
@@ -6442,7 +6499,7 @@
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -6514,7 +6571,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -6586,7 +6643,7 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
@@ -6658,7 +6715,7 @@
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K86" s="5" t="inlineStr">
@@ -6730,7 +6787,7 @@
       </c>
       <c r="J87" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K87" s="5" t="inlineStr">
@@ -6802,7 +6859,7 @@
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K88" s="5" t="inlineStr">
@@ -6874,7 +6931,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -6946,7 +7003,7 @@
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K90" s="5" t="inlineStr">
@@ -7018,7 +7075,7 @@
       </c>
       <c r="J91" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K91" s="5" t="inlineStr">
@@ -7090,7 +7147,7 @@
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K92" s="5" t="inlineStr">
@@ -7162,7 +7219,7 @@
       </c>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K93" s="5" t="inlineStr">
@@ -7234,7 +7291,7 @@
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -7298,7 +7355,7 @@
       </c>
       <c r="J95" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K95" s="5" t="inlineStr">
@@ -7370,7 +7427,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
@@ -7442,7 +7499,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -7514,7 +7571,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -7586,7 +7643,7 @@
       </c>
       <c r="J99" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K99" s="5" t="inlineStr">
@@ -7658,7 +7715,7 @@
       </c>
       <c r="J100" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K100" s="5" t="inlineStr">
@@ -7730,7 +7787,7 @@
       </c>
       <c r="J101" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
@@ -7802,7 +7859,7 @@
       </c>
       <c r="J102" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K102" s="5" t="inlineStr">
@@ -7874,7 +7931,7 @@
       </c>
       <c r="J103" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K103" s="5" t="inlineStr">
@@ -7946,7 +8003,7 @@
       </c>
       <c r="J104" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K104" s="5" t="inlineStr">
@@ -8018,7 +8075,7 @@
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
@@ -8090,7 +8147,7 @@
       </c>
       <c r="J106" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr">
@@ -8162,7 +8219,7 @@
       </c>
       <c r="J107" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K107" s="5" t="inlineStr">
@@ -8234,7 +8291,7 @@
       </c>
       <c r="J108" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K108" s="2" t="inlineStr">
@@ -8306,7 +8363,7 @@
       </c>
       <c r="J109" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K109" s="5" t="inlineStr">
@@ -8378,7 +8435,7 @@
       </c>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K110" s="5" t="inlineStr">
@@ -8450,7 +8507,7 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K111" s="2" t="inlineStr">
@@ -8522,7 +8579,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr">
@@ -8594,7 +8651,7 @@
       </c>
       <c r="J113" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K113" s="5" t="inlineStr">
@@ -8666,7 +8723,7 @@
       </c>
       <c r="J114" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K114" s="5" t="inlineStr">
@@ -8738,7 +8795,7 @@
       </c>
       <c r="J115" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K115" s="2" t="inlineStr">
@@ -8810,7 +8867,7 @@
       </c>
       <c r="J116" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K116" s="2" t="inlineStr">
@@ -8882,7 +8939,7 @@
       </c>
       <c r="J117" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K117" s="5" t="inlineStr">
@@ -8954,7 +9011,7 @@
       </c>
       <c r="J118" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K118" s="5" t="inlineStr">
@@ -9026,7 +9083,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr">
@@ -9098,7 +9155,7 @@
       </c>
       <c r="J120" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K120" s="2" t="inlineStr">
@@ -9170,7 +9227,7 @@
       </c>
       <c r="J121" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K121" s="5" t="inlineStr">
@@ -9242,7 +9299,7 @@
       </c>
       <c r="J122" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K122" s="5" t="inlineStr">
@@ -9314,7 +9371,7 @@
       </c>
       <c r="J123" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K123" s="5" t="inlineStr">
@@ -9386,7 +9443,7 @@
       </c>
       <c r="J124" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K124" s="5" t="inlineStr">
@@ -9458,7 +9515,7 @@
       </c>
       <c r="J125" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K125" s="5" t="inlineStr">
@@ -9530,7 +9587,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K126" s="2" t="inlineStr">
@@ -9602,7 +9659,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr">
@@ -9674,7 +9731,7 @@
       </c>
       <c r="J128" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K128" s="5" t="inlineStr">
@@ -9746,7 +9803,7 @@
       </c>
       <c r="J129" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K129" s="5" t="inlineStr">
@@ -9818,7 +9875,7 @@
       </c>
       <c r="J130" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K130" s="2" t="inlineStr">
@@ -9890,7 +9947,7 @@
       </c>
       <c r="J131" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K131" s="5" t="inlineStr">
@@ -9962,7 +10019,7 @@
       </c>
       <c r="J132" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K132" s="5" t="inlineStr">
@@ -10034,7 +10091,7 @@
       </c>
       <c r="J133" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K133" s="5" t="inlineStr">
@@ -10106,7 +10163,7 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K134" s="2" t="inlineStr">
@@ -10178,7 +10235,7 @@
       </c>
       <c r="J135" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K135" s="5" t="inlineStr">
@@ -10238,7 +10295,7 @@
       </c>
       <c r="J136" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K136" s="5" t="inlineStr">
@@ -10298,7 +10355,7 @@
       </c>
       <c r="J137" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K137" s="5" t="inlineStr">
@@ -10358,7 +10415,7 @@
       </c>
       <c r="J138" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K138" s="5" t="inlineStr">
@@ -10418,7 +10475,7 @@
       </c>
       <c r="J139" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K139" s="5" t="inlineStr">
@@ -10478,7 +10535,7 @@
       </c>
       <c r="J140" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K140" s="5" t="inlineStr">
@@ -10538,7 +10595,7 @@
       </c>
       <c r="J141" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K141" s="5" t="inlineStr">
@@ -10598,7 +10655,7 @@
       </c>
       <c r="J142" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K142" s="5" t="inlineStr">
@@ -10658,7 +10715,7 @@
       </c>
       <c r="J143" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K143" s="5" t="inlineStr">
@@ -10718,7 +10775,7 @@
       </c>
       <c r="J144" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K144" s="5" t="inlineStr">
@@ -10778,7 +10835,7 @@
       </c>
       <c r="J145" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K145" s="5" t="inlineStr">
@@ -10838,7 +10895,7 @@
       </c>
       <c r="J146" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K146" s="5" t="inlineStr">
@@ -10898,7 +10955,7 @@
       </c>
       <c r="J147" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K147" s="5" t="inlineStr">
@@ -10970,7 +11027,7 @@
       </c>
       <c r="J148" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K148" s="2" t="inlineStr">
@@ -11042,7 +11099,7 @@
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K149" s="2" t="inlineStr">
@@ -11114,7 +11171,7 @@
       </c>
       <c r="J150" s="5" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="K150" s="5" t="inlineStr">
@@ -11140,6 +11197,23 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:N150"/>
+  <conditionalFormatting sqref="I2:I150">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>$I2="Passed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="0">
+      <formula>$I2="Fail" OR $I2="Failed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="0">
+      <formula>$I2="Not Run"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="0">
+      <formula>$I2="Blocked" OR $I2="Retest"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="0">
+      <formula>$I2="Skipped"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(qa): kolom Pembuat Test & Link Bug di output generator + override CLI run-date/environment
- Generator (scripts/generate-qa-test-cases.py):
  - Kolom baru di tracker CSV & XLSX: "Pembuat Test" (default Tim QA, editable
    per baris) dan "Link Bug" (kosong, diisi QA saat ada defect)
  - RUN_DATE_DEFAULT & ENVIRONMENT_DEFAULT kini bisa di-override via argumen
    CLI --run-date / --environment (prioritas CLI > env QA_RUN_DATE /
    QA_ENVIRONMENT > default) — env QA_RUN_DATE tetap dipakai check-qa-sync
- Output diregenerasi dari QA Test Plan (137 TC + 12 RG = 149 test case):
  - qa-test-cases-tracker.csv & qa-test-cases.xlsx dengan kolom baru;
    status 149 test case yang sudah diisi dipertahankan
- Verifikasi: gate check-qa-sync [OK] (5 file sinkron), status terjaga
</commit_message>
<xml_diff>
--- a/qa-test-cases.xlsx
+++ b/qa-test-cases.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$N$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$P$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N150"/>
+  <dimension ref="A1:P150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -542,9 +542,11 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="60" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
-    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,15 +607,25 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Pembuat Test</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Link Bug</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Langkah</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Hasil Diharapkan</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Preconditions</t>
         </is>
@@ -675,17 +687,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Buka aplikasi sebagai Rina</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Top bar 64px (logo+nama, search, notif, profil), sidebar 280px 9 modul + "+ Buat Jurnal", bottom bar 32px (versi, periode, koneksi)</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -747,17 +765,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Klik tiap item sidebar</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Rute berfungsi, item aktif bg-primary/10 + border-left 3px, URL berubah, lazy loading tanpa error</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -819,17 +843,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Klik toggle</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>280px ↔ 64px (ikon saja); state tersimpan; hover bg-slate-100</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -891,17 +921,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>Klik "Laporan Lain"</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>Expand/collapse submenu; item anak tampil</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -963,17 +999,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Resize 1440 / 768 / 375 / 320px</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>Desktop penuh; tablet sidebar collapse; mobile drawer; tidak ada horizontal scroll</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="P6" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1035,17 +1077,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Inspeksi CSS</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>Biru #2596BE (primary), Inter + JetBrains Mono aktif</t>
         </is>
       </c>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1107,17 +1155,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Klik "+ Buat Jurnal" di sidebar</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>Navigasi ke form jurnal baru, periode = periode aktif</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1179,17 +1233,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Buka modul COA</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>Tree dengan 5 tipe akun, indentasi bertingkat, expand/collapse per grup, ikon + badge tipe, baris berisi kode+nama+saldo IDR</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1251,17 +1311,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Bandingkan saldo tree vs buku besar</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Kas Besar = 87.000.000; akun header (1-1000) = jumlah anak 557jt</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1323,17 +1389,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>Reset data tanpa template, buka COA</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>"Chart of Account masih kosong. Buat akun pertama Anda." + CTA Muat Template</t>
         </is>
       </c>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>COA kosong (belum dimuat template)</t>
         </is>
@@ -1395,17 +1467,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr"/>
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>Simulasi delay API</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>Skeleton 5 baris saat loading</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="P12" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1467,17 +1545,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Form tambah: 1-1500 Kas Kecil, asset, debit, parent 1-1000</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>201; akun muncul di tree di bawah parent, saldo 0</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1539,17 +1623,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr"/>
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>Buat akun kode 1-1100</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>Toast 409 "Kode akun sudah digunakan"; form tetap terbuka</t>
         </is>
       </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="P14" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1611,17 +1701,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr"/>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>Kode abc / 11x00</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
         <is>
           <t>"Format kode tidak valid" (422 INVALID_CODE_FORMAT)</t>
         </is>
       </c>
-      <c r="N15" s="6" t="inlineStr">
+      <c r="P15" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1683,17 +1779,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr"/>
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>Coba hapus 1-1000 (punya 4 anak aktif)</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>Diblokir 409 "Akun induk tidak bisa dihapus jika memiliki sub-akun aktif"</t>
         </is>
       </c>
-      <c r="N16" s="6" t="inlineStr">
+      <c r="P16" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1755,17 +1857,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>Coba hapus 1-1100 (saldo 87jt)</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>Warning konfirmasi; hanya bisa dinonaktifkan (409 ACCOUNT_HAS_BALANCE)</t>
         </is>
       </c>
-      <c r="N17" s="6" t="inlineStr">
+      <c r="P17" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1827,17 +1935,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr"/>
+      <c r="N18" s="6" t="inlineStr">
         <is>
           <t>Deactivate 1-1400</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>Status non-aktif; tidak muncul di dropdown akun jurnal</t>
         </is>
       </c>
-      <c r="N18" s="6" t="inlineStr">
+      <c r="P18" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1899,17 +2013,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr"/>
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>Buka form edit akun</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>Tidak ada field saldo; saldo hanya berubah via jurnal</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="P19" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -1971,17 +2091,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Klik "Muat Template UKM PSAK" (COA kosong)</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>≥40 akun standar ter-muat; toast "Template berhasil dimuat"; tree menampilkan akun baru</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>COA kosong (belum dimuat template)</t>
         </is>
@@ -2043,17 +2169,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr"/>
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>COA terisi → muat template</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr">
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>Dialog konfirmasi replace vs merge; replace tanpa konfirmasi → 409 ACCOUNTS_EXIST</t>
         </is>
       </c>
-      <c r="N21" s="6" t="inlineStr">
+      <c r="P21" s="6" t="inlineStr">
         <is>
           <t>COA sudah terisi akun</t>
         </is>
@@ -2115,17 +2247,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr">
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr"/>
+      <c r="N22" s="6" t="inlineStr">
         <is>
           <t>Klik export → XLSX</t>
         </is>
       </c>
-      <c r="M22" s="6" t="inlineStr">
+      <c r="O22" s="6" t="inlineStr">
         <is>
           <t>File chart-of-accounts.xlsx terunduh; header rapi; nilai angka</t>
         </is>
       </c>
-      <c r="N22" s="6" t="inlineStr">
+      <c r="P22" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2187,17 +2325,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr"/>
+      <c r="N23" s="6" t="inlineStr">
         <is>
           <t>Upload XLSX berisi 1 baris duplikat</t>
         </is>
       </c>
-      <c r="M23" s="6" t="inlineStr">
+      <c r="O23" s="6" t="inlineStr">
         <is>
           <t>Laporan { imported, failed, errors: [{row, code, message}] }; baris gagal tidak menggagalkan seluruh import; preview sebelum konfirmasi</t>
         </is>
       </c>
-      <c r="N23" s="6" t="inlineStr">
+      <c r="P23" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2259,17 +2403,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>Buka "+ Buat Jurnal"</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Field: tanggal, no. bukti (auto), deskripsi, baris (dropdown akun, deskripsi, debit, kredit); akun dropdown hanya aktif</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2331,17 +2481,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>Ketik debit 10jt baris 1</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>Footer total live; debit≠kredit → pesan "Total debit (10.000.000) dan kredit (0) harus sama. Selisih: 10.000.000"</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="P25" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2403,17 +2559,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>Form belum balance</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Tombol Posting disabled</t>
         </is>
       </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="P26" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2475,17 +2637,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr">
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr"/>
+      <c r="N27" s="6" t="inlineStr">
         <is>
           <t>Isi debit &amp; kredit di baris sama</t>
         </is>
       </c>
-      <c r="M27" s="6" t="inlineStr">
+      <c r="O27" s="6" t="inlineStr">
         <is>
           <t>Ditolak (422 LINE_BOTH_SIDES); salah satu wajib 0</t>
         </is>
       </c>
-      <c r="N27" s="6" t="inlineStr">
+      <c r="P27" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2547,17 +2715,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr">
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr"/>
+      <c r="N28" s="6" t="inlineStr">
         <is>
           <t>Ketik debit −5.000</t>
         </is>
       </c>
-      <c r="M28" s="6" t="inlineStr">
+      <c r="O28" s="6" t="inlineStr">
         <is>
           <t>Ditolak (422 LINE_NEGATIVE_AMOUNT)</t>
         </is>
       </c>
-      <c r="N28" s="6" t="inlineStr">
+      <c r="P28" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2619,17 +2793,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr">
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr"/>
+      <c r="N29" s="6" t="inlineStr">
         <is>
           <t>Simpan dengan 1 baris saja</t>
         </is>
       </c>
-      <c r="M29" s="6" t="inlineStr">
+      <c r="O29" s="6" t="inlineStr">
         <is>
           <t>Gagal (422 JOURNAL_NO_LINES); minimal 1 debit + 1 kredit</t>
         </is>
       </c>
-      <c r="N29" s="6" t="inlineStr">
+      <c r="P29" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2691,17 +2871,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L30" s="6" t="inlineStr">
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr"/>
+      <c r="N30" s="6" t="inlineStr">
         <is>
           <t>Klik + baris / hapus baris</t>
         </is>
       </c>
-      <c r="M30" s="6" t="inlineStr">
+      <c r="O30" s="6" t="inlineStr">
         <is>
           <t>Baris dinamis bertambah/berkurang; total live ter-update</t>
         </is>
       </c>
-      <c r="N30" s="6" t="inlineStr">
+      <c r="P30" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2763,17 +2949,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L31" s="6" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr"/>
+      <c r="N31" s="6" t="inlineStr">
         <is>
           <t>Ketik 15000000</t>
         </is>
       </c>
-      <c r="M31" s="6" t="inlineStr">
+      <c r="O31" s="6" t="inlineStr">
         <is>
           <t>Muncul 15.000.000 otomatis; Tab/Enter menambah baris</t>
         </is>
       </c>
-      <c r="N31" s="6" t="inlineStr">
+      <c r="P31" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2835,17 +3027,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L32" s="6" t="inlineStr">
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr"/>
+      <c r="N32" s="6" t="inlineStr">
         <is>
           <t>Cari akun yang di-deactivate</t>
         </is>
       </c>
-      <c r="M32" s="6" t="inlineStr">
+      <c r="O32" s="6" t="inlineStr">
         <is>
           <t>Tidak tampil di dropdown</t>
         </is>
       </c>
-      <c r="N32" s="6" t="inlineStr">
+      <c r="P32" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2907,17 +3105,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>Buka form baru periode 2026-03 prefix BKM</t>
         </is>
       </c>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="O33" s="4" t="inlineStr">
         <is>
           <t>BKM-2026-03-0009 (dari GET /journals/next-number); format {{PREFIX}}-{{TAHUN}}-{{BULAN}}-{{NOMOR}}</t>
         </is>
       </c>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="P33" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -2979,17 +3183,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L34" s="6" t="inlineStr">
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr"/>
+      <c r="N34" s="6" t="inlineStr">
         <is>
           <t>Ketik BKM-2026-03-0001 manual</t>
         </is>
       </c>
-      <c r="M34" s="6" t="inlineStr">
+      <c r="O34" s="6" t="inlineStr">
         <is>
           <t>Error "Nomor bukti sudah digunakan" (409 TRANSACTION_NUMBER_DUPLICATE)</t>
         </is>
       </c>
-      <c r="N34" s="6" t="inlineStr">
+      <c r="P34" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3051,17 +3261,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L35" s="6" t="inlineStr">
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr"/>
+      <c r="N35" s="6" t="inlineStr">
         <is>
           <t>Next-number periode 2026-04</t>
         </is>
       </c>
-      <c r="M35" s="6" t="inlineStr">
+      <c r="O35" s="6" t="inlineStr">
         <is>
           <t>Mulai dari -0001 (nomor tidak nyambung antar periode)</t>
         </is>
       </c>
-      <c r="N35" s="6" t="inlineStr">
+      <c r="P35" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3123,17 +3339,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>Isi jurnal balance → Simpan Draft</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="O36" s="4" t="inlineStr">
         <is>
           <t>Status draft; saldo tidak berubah; tidak muncul di laporan; toast "Jurnal disimpan sebagai draft"</t>
         </is>
       </c>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="P36" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3195,17 +3417,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>Buat &amp; posting: Kas 10jt / Pendapatan 10jt (BKM-2026-03-0009)</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="O37" s="4" t="inlineStr">
         <is>
           <t>Status posted; Kas 87→97jt; Pendapatan 155→165jt (cek COA &amp; dashboard); toast "Jurnal berhasil diposting"</t>
         </is>
       </c>
-      <c r="N37" s="4" t="inlineStr">
+      <c r="P37" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3267,17 +3495,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>Buat jurnal tgl 2026-02-15 (Februari tertutup) → Posting</t>
         </is>
       </c>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>Diblokir "Periode Februari 2026 sudah ditutup" (422 PERIOD_CLOSED)</t>
         </is>
       </c>
-      <c r="N38" s="4" t="inlineStr">
+      <c r="P38" s="4" t="inlineStr">
         <is>
           <t>Reset data seed; periode Februari 2026 tertutup</t>
         </is>
@@ -3339,17 +3573,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L39" s="4" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>Edit draft JNL-07 → simpan; hapus draft JNL-06</t>
         </is>
       </c>
-      <c r="M39" s="4" t="inlineStr">
+      <c r="O39" s="4" t="inlineStr">
         <is>
           <t>Edit berhasil tanpa ubah saldo; hapus dengan dialog "Yakin ingin menghapus jurnal ini?" → hilang dari daftar</t>
         </is>
       </c>
-      <c r="N39" s="4" t="inlineStr">
+      <c r="P39" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3411,17 +3651,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L40" s="6" t="inlineStr">
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr"/>
+      <c r="N40" s="6" t="inlineStr">
         <is>
           <t>Buka jurnal posted JNL-01</t>
         </is>
       </c>
-      <c r="M40" s="6" t="inlineStr">
+      <c r="O40" s="6" t="inlineStr">
         <is>
           <t>Form terkunci (disabled); tombol edit disabled + tooltip</t>
         </is>
       </c>
-      <c r="N40" s="6" t="inlineStr">
+      <c r="P40" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3483,17 +3729,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L41" s="6" t="inlineStr">
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr"/>
+      <c r="N41" s="6" t="inlineStr">
         <is>
           <t>Klik Posting 2× cepat</t>
         </is>
       </c>
-      <c r="M41" s="6" t="inlineStr">
+      <c r="O41" s="6" t="inlineStr">
         <is>
           <t>Tombol disabled + "Menyimpan..."; hanya 1 jurnal dibuat</t>
         </is>
       </c>
-      <c r="N41" s="6" t="inlineStr">
+      <c r="P41" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3555,17 +3807,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L42" s="4" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="4" t="inlineStr">
         <is>
           <t>Buka modul Jurnal</t>
         </is>
       </c>
-      <c r="M42" s="4" t="inlineStr">
+      <c r="O42" s="4" t="inlineStr">
         <is>
           <t>Kolom Tgl/No. Bukti/Keterangan (line-item dikelompokkan)/Debit/Kredit; badge status Draft(slate)/Posted(green)/Reversed(red)</t>
         </is>
       </c>
-      <c r="N42" s="4" t="inlineStr">
+      <c r="P42" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3627,17 +3885,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L43" s="4" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="4" t="inlineStr">
         <is>
           <t>Periksa footer daftar</t>
         </is>
       </c>
-      <c r="M43" s="4" t="inlineStr">
+      <c r="O43" s="4" t="inlineStr">
         <is>
           <t>Total debit = total kredit = 98.000.000 (seed), selisih 0</t>
         </is>
       </c>
-      <c r="N43" s="4" t="inlineStr">
+      <c r="P43" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3699,17 +3963,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L44" s="6" t="inlineStr">
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr"/>
+      <c r="N44" s="6" t="inlineStr">
         <is>
           <t>Klik expand jurnal</t>
         </is>
       </c>
-      <c r="M44" s="6" t="inlineStr">
+      <c r="O44" s="6" t="inlineStr">
         <is>
           <t>Detail + line-items + lampiran (placeholder); aksi Lihat Detail/Edit/Posting/Reverse/Hapus sesuai status</t>
         </is>
       </c>
-      <c r="N44" s="6" t="inlineStr">
+      <c r="P44" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3771,17 +4041,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L45" s="6" t="inlineStr">
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr"/>
+      <c r="N45" s="6" t="inlineStr">
         <is>
           <t>Filter sehingga kosong / entitas baru</t>
         </is>
       </c>
-      <c r="M45" s="6" t="inlineStr">
+      <c r="O45" s="6" t="inlineStr">
         <is>
           <t>"Belum ada transaksi. Mulai catat jurnal pertama Anda!" + CTA</t>
         </is>
       </c>
-      <c r="N45" s="6" t="inlineStr">
+      <c r="P45" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3843,17 +4119,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L46" s="6" t="inlineStr">
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr"/>
+      <c r="N46" s="6" t="inlineStr">
         <is>
           <t>Buka detail JNL-01</t>
         </is>
       </c>
-      <c r="M46" s="6" t="inlineStr">
+      <c r="O46" s="6" t="inlineStr">
         <is>
           <t>Riwayat create (Rina 09:10), post (Rina 09:12) dengan user+timestamp; edit draft menambah entry update</t>
         </is>
       </c>
-      <c r="N46" s="6" t="inlineStr">
+      <c r="P46" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3915,17 +4197,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L47" s="6" t="inlineStr">
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr"/>
+      <c r="N47" s="6" t="inlineStr">
         <is>
           <t>Buka tab lain, edit draft, lalu edit lagi dengan versi lama (simulasi 409)</t>
         </is>
       </c>
-      <c r="M47" s="6" t="inlineStr">
+      <c r="O47" s="6" t="inlineStr">
         <is>
           <t>409 DATA_CONFLICT "Data sudah diubah oleh pengguna lain. Muat ulang halaman."</t>
         </is>
       </c>
-      <c r="N47" s="6" t="inlineStr">
+      <c r="P47" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -3987,17 +4275,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L48" s="4" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="4" t="inlineStr">
         <is>
           <t>Buka Buku Besar → 1-1100, periode 2026-03</t>
         </is>
       </c>
-      <c r="M48" s="4" t="inlineStr">
+      <c r="O48" s="4" t="inlineStr">
         <is>
           <t>Header kode+nama+periode; 4 baris + Saldo Awal 60jt + Saldo Akhir 87jt; saldo berjalan: 85 / 75 / 72 / 87</t>
         </is>
       </c>
-      <c r="N48" s="4" t="inlineStr">
+      <c r="P48" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4059,17 +4353,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L49" s="4" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="4" t="inlineStr">
         <is>
           <t>Periksa baris pertama &amp; terakhir</t>
         </is>
       </c>
-      <c r="M49" s="4" t="inlineStr">
+      <c r="O49" s="4" t="inlineStr">
         <is>
           <t>Baris "Saldo Awal" (60jt) &amp; footer "Saldo Akhir" (87jt)</t>
         </is>
       </c>
-      <c r="N49" s="4" t="inlineStr">
+      <c r="P49" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4131,17 +4431,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L50" s="4" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="4" t="inlineStr">
         <is>
           <t>Cek jurnal draft JNL-06/07 di semua buku besar</t>
         </is>
       </c>
-      <c r="M50" s="4" t="inlineStr">
+      <c r="O50" s="4" t="inlineStr">
         <is>
           <t>Tidak muncul (draft tidak mempengaruhi buku besar)</t>
         </is>
       </c>
-      <c r="N50" s="4" t="inlineStr">
+      <c r="P50" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4203,17 +4509,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L51" s="6" t="inlineStr">
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr"/>
+      <c r="N51" s="6" t="inlineStr">
         <is>
           <t>Klik prev/next periode</t>
         </is>
       </c>
-      <c r="M51" s="6" t="inlineStr">
+      <c r="O51" s="6" t="inlineStr">
         <is>
           <t>Periode berganti, data re-fetch; periode Jan/Feb tetap bisa dibaca</t>
         </is>
       </c>
-      <c r="N51" s="6" t="inlineStr">
+      <c r="P51" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4275,17 +4587,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L52" s="6" t="inlineStr">
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr"/>
+      <c r="N52" s="6" t="inlineStr">
         <is>
           <t>Klik ref BKM-2026-03-0001</t>
         </is>
       </c>
-      <c r="M52" s="6" t="inlineStr">
+      <c r="O52" s="6" t="inlineStr">
         <is>
           <t>Buka detail jurnal sumber</t>
         </is>
       </c>
-      <c r="N52" s="6" t="inlineStr">
+      <c r="P52" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4347,17 +4665,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L53" s="6" t="inlineStr">
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr"/>
+      <c r="N53" s="6" t="inlineStr">
         <is>
           <t>Buka /ledger rekap</t>
         </is>
       </c>
-      <c r="M53" s="6" t="inlineStr">
+      <c r="O53" s="6" t="inlineStr">
         <is>
           <t>Semua akun dengan opening, total D/K, closing; header tidak muncul</t>
         </is>
       </c>
-      <c r="N53" s="6" t="inlineStr">
+      <c r="P53" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4419,17 +4743,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L54" s="4" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="4" t="inlineStr">
         <is>
           <t>Rentang 01–10 Mar</t>
         </is>
       </c>
-      <c r="M54" s="4" t="inlineStr">
+      <c r="O54" s="4" t="inlineStr">
         <is>
           <t>Hanya jurnal JNL-01/02/03; footer agregat mengikuti filter</t>
         </is>
       </c>
-      <c r="N54" s="4" t="inlineStr">
+      <c r="P54" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4491,17 +4821,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L55" s="6" t="inlineStr">
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr"/>
+      <c r="N55" s="6" t="inlineStr">
         <is>
           <t>status=posted,draft</t>
         </is>
       </c>
-      <c r="M55" s="6" t="inlineStr">
+      <c r="O55" s="6" t="inlineStr">
         <is>
           <t>5 posted + 2 draft tampil; reversed tidak</t>
         </is>
       </c>
-      <c r="N55" s="6" t="inlineStr">
+      <c r="P55" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4563,17 +4899,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L56" s="6" t="inlineStr">
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr"/>
+      <c r="N56" s="6" t="inlineStr">
         <is>
           <t>accountId=1-1100</t>
         </is>
       </c>
-      <c r="M56" s="6" t="inlineStr">
+      <c r="O56" s="6" t="inlineStr">
         <is>
           <t>Hanya jurnal yang menyentuh Kas Besar (JNL-01,02,03,04)</t>
         </is>
       </c>
-      <c r="N56" s="6" t="inlineStr">
+      <c r="P56" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4635,17 +4977,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L57" s="6" t="inlineStr">
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr"/>
+      <c r="N57" s="6" t="inlineStr">
         <is>
           <t>status=posted &amp; keyword=sewa</t>
         </is>
       </c>
-      <c r="M57" s="6" t="inlineStr">
+      <c r="O57" s="6" t="inlineStr">
         <is>
           <t>Hanya JNL-02 (BKK-0002 sewa, posted)</t>
         </is>
       </c>
-      <c r="N57" s="6" t="inlineStr">
+      <c r="P57" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4707,17 +5055,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L58" s="6" t="inlineStr">
+      <c r="L58" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M58" s="5" t="inlineStr"/>
+      <c r="N58" s="6" t="inlineStr">
         <is>
           <t>Ketik "sewa"</t>
         </is>
       </c>
-      <c r="M58" s="6" t="inlineStr">
+      <c r="O58" s="6" t="inlineStr">
         <is>
           <t>Setelah 300ms hasil = 1 jurnal; empty state "Tidak ditemukan jurnal dengan kata kunci 'xyz'"</t>
         </is>
       </c>
-      <c r="N58" s="6" t="inlineStr">
+      <c r="P58" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4779,17 +5133,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L59" s="6" t="inlineStr">
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M59" s="5" t="inlineStr"/>
+      <c r="N59" s="6" t="inlineStr">
         <is>
           <t>Filter lalu refresh</t>
         </is>
       </c>
-      <c r="M59" s="6" t="inlineStr">
+      <c r="O59" s="6" t="inlineStr">
         <is>
           <t>Filter tersimpan di URL (?period=&amp;status=), re-render sama</t>
         </is>
       </c>
-      <c r="N59" s="6" t="inlineStr">
+      <c r="P59" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4851,17 +5211,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L60" s="6" t="inlineStr">
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M60" s="5" t="inlineStr"/>
+      <c r="N60" s="6" t="inlineStr">
         <is>
           <t>Ketik "bkm"</t>
         </is>
       </c>
-      <c r="M60" s="6" t="inlineStr">
+      <c r="O60" s="6" t="inlineStr">
         <is>
           <t>Hasil jurnal (no. bukti) &amp; akun (kode/nama); terkelompok per tipe; klik → navigasi</t>
         </is>
       </c>
-      <c r="N60" s="6" t="inlineStr">
+      <c r="P60" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4923,17 +5289,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L61" s="6" t="inlineStr">
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="inlineStr"/>
+      <c r="N61" s="6" t="inlineStr">
         <is>
           <t>Ketik "zzz"</t>
         </is>
       </c>
-      <c r="M61" s="6" t="inlineStr">
+      <c r="O61" s="6" t="inlineStr">
         <is>
           <t>"Tidak ditemukan hasil untuk 'zzz'"</t>
         </is>
       </c>
-      <c r="N61" s="6" t="inlineStr">
+      <c r="P61" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -4995,17 +5367,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L62" s="4" t="inlineStr">
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="4" t="inlineStr">
         <is>
           <t>Pengaturan → Periode</t>
         </is>
       </c>
-      <c r="M62" s="4" t="inlineStr">
+      <c r="O62" s="4" t="inlineStr">
         <is>
           <t>Bulan/tahun/rentang/status; Maret aktif terbuka; Jan &amp; Feb terkunci; badge "Terkunci"</t>
         </is>
       </c>
-      <c r="N62" s="4" t="inlineStr">
+      <c r="P62" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5067,17 +5445,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L63" s="4" t="inlineStr">
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="4" t="inlineStr">
         <is>
           <t>Klik activate April</t>
         </is>
       </c>
-      <c r="M63" s="4" t="inlineStr">
+      <c r="O63" s="4" t="inlineStr">
         <is>
           <t>April jadi aktif; Maret tidak; default entri jurnal baru = April</t>
         </is>
       </c>
-      <c r="N63" s="4" t="inlineStr">
+      <c r="P63" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5139,17 +5523,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L64" s="4" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="4" t="inlineStr">
         <is>
           <t>Tutup Maret dengan dialog</t>
         </is>
       </c>
-      <c r="M64" s="4" t="inlineStr">
+      <c r="O64" s="4" t="inlineStr">
         <is>
           <t>Dialog konfirmasi + pilihan post-all / delete-all / keep; handledDrafts sesuai aksi</t>
         </is>
       </c>
-      <c r="N64" s="4" t="inlineStr">
+      <c r="P64" s="4" t="inlineStr">
         <is>
           <t>Reset data seed; Maret 2026 masih punya 2 jurnal draft</t>
         </is>
@@ -5211,17 +5601,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L65" s="6" t="inlineStr">
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M65" s="5" t="inlineStr"/>
+      <c r="N65" s="6" t="inlineStr">
         <is>
           <t>Maret masih punya 2 draft → tutup tanpa pilih aksi</t>
         </is>
       </c>
-      <c r="M65" s="6" t="inlineStr">
+      <c r="O65" s="6" t="inlineStr">
         <is>
           <t>422 DRAFT_ACTION_REQUIRED "Masih ada jurnal draft; pilih aksi terlebih dahulu"</t>
         </is>
       </c>
-      <c r="N65" s="6" t="inlineStr">
+      <c r="P65" s="6" t="inlineStr">
         <is>
           <t>Reset data seed; Maret 2026 masih punya 2 jurnal draft</t>
         </is>
@@ -5283,17 +5679,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L66" s="4" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="4" t="inlineStr">
         <is>
           <t>Tutup Maret → buat/posting jurnal Maret</t>
         </is>
       </c>
-      <c r="M66" s="4" t="inlineStr">
+      <c r="O66" s="4" t="inlineStr">
         <is>
           <t>Diblokir di semua modul dengan warning jelas; laporan Maret tetap bisa dibaca</t>
         </is>
       </c>
-      <c r="N66" s="4" t="inlineStr">
+      <c r="P66" s="4" t="inlineStr">
         <is>
           <t>Reset data seed; Maret 2026 sudah ditutup</t>
         </is>
@@ -5355,17 +5757,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L67" s="6" t="inlineStr">
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M67" s="5" t="inlineStr"/>
+      <c r="N67" s="6" t="inlineStr">
         <is>
           <t>Tutup periode yang sudah tertutup</t>
         </is>
       </c>
-      <c r="M67" s="6" t="inlineStr">
+      <c r="O67" s="6" t="inlineStr">
         <is>
           <t>409 PERIOD_ALREADY_CLOSED</t>
         </is>
       </c>
-      <c r="N67" s="6" t="inlineStr">
+      <c r="P67" s="6" t="inlineStr">
         <is>
           <t>Reset data seed; periode Maret 2026 sudah ditutup</t>
         </is>
@@ -5427,17 +5835,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L68" s="4" t="inlineStr">
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr"/>
+      <c r="N68" s="4" t="inlineStr">
         <is>
           <t>Ganti periode di sidebar → buka Laba Rugi/Neraca/Buku Besar/Dashboard</t>
         </is>
       </c>
-      <c r="M68" s="4" t="inlineStr">
+      <c r="O68" s="4" t="inlineStr">
         <is>
           <t>Semua modul re-fetch &amp; re-render sesuai periode; URL ?period=2026-03; bisa di-share</t>
         </is>
       </c>
-      <c r="N68" s="4" t="inlineStr">
+      <c r="P68" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5499,17 +5913,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L69" s="4" t="inlineStr">
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr"/>
+      <c r="N69" s="4" t="inlineStr">
         <is>
           <t>Buka Dashboard</t>
         </is>
       </c>
-      <c r="M69" s="4" t="inlineStr">
+      <c r="O69" s="4" t="inlineStr">
         <is>
           <t>Total Aset 557jt, Total Utang 150jt, Total Modal 363jt, Laba Bruto 44jt (IDR)</t>
         </is>
       </c>
-      <c r="N69" s="4" t="inlineStr">
+      <c r="P69" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5571,17 +5991,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L70" s="6" t="inlineStr">
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr"/>
+      <c r="N70" s="6" t="inlineStr">
         <is>
           <t>Periksa kartu</t>
         </is>
       </c>
-      <c r="M70" s="6" t="inlineStr">
+      <c r="O70" s="6" t="inlineStr">
         <is>
           <t>Panah ▲/▼ + delta %; utang naik = merah, aset naik = hijau</t>
         </is>
       </c>
-      <c r="N70" s="6" t="inlineStr">
+      <c r="P70" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5643,17 +6069,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L71" s="6" t="inlineStr">
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M71" s="5" t="inlineStr"/>
+      <c r="N71" s="6" t="inlineStr">
         <is>
           <t>Klik kartu Total Aset</t>
         </is>
       </c>
-      <c r="M71" s="6" t="inlineStr">
+      <c r="O71" s="6" t="inlineStr">
         <is>
           <t>Navigasi ke Neraca</t>
         </is>
       </c>
-      <c r="N71" s="6" t="inlineStr">
+      <c r="P71" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5715,17 +6147,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L72" s="6" t="inlineStr">
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M72" s="5" t="inlineStr"/>
+      <c r="N72" s="6" t="inlineStr">
         <is>
           <t>Periksa grafik</t>
         </is>
       </c>
-      <c r="M72" s="6" t="inlineStr">
+      <c r="O72" s="6" t="inlineStr">
         <is>
           <t>Bar chart Okt 2025 – Mar 2026 (Recharts, lazy-loaded)</t>
         </is>
       </c>
-      <c r="N72" s="6" t="inlineStr">
+      <c r="P72" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5787,17 +6225,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L73" s="6" t="inlineStr">
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M73" s="5" t="inlineStr"/>
+      <c r="N73" s="6" t="inlineStr">
         <is>
           <t>Periksa panel</t>
         </is>
       </c>
-      <c r="M73" s="6" t="inlineStr">
+      <c r="O73" s="6" t="inlineStr">
         <is>
           <t>5 jurnal terbaru + link "Lihat Semua" → modul Jurnal</t>
         </is>
       </c>
-      <c r="N73" s="6" t="inlineStr">
+      <c r="P73" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5859,17 +6303,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L74" s="6" t="inlineStr">
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr"/>
+      <c r="N74" s="6" t="inlineStr">
         <is>
           <t>Periksa panel alert</t>
         </is>
       </c>
-      <c r="M74" s="6" t="inlineStr">
+      <c r="O74" s="6" t="inlineStr">
         <is>
           <t>2 alert: jurnal draft belum diposting (count 2), periode Februari belum ditutup (info)</t>
         </is>
       </c>
-      <c r="N74" s="6" t="inlineStr">
+      <c r="P74" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -5931,17 +6381,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L75" s="6" t="inlineStr">
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M75" s="5" t="inlineStr"/>
+      <c r="N75" s="6" t="inlineStr">
         <is>
           <t>Klik alert draft jurnal</t>
         </is>
       </c>
-      <c r="M75" s="6" t="inlineStr">
+      <c r="O75" s="6" t="inlineStr">
         <is>
           <t>Navigasi ke tempat perbaikan (modul Jurnal filter draft)</t>
         </is>
       </c>
-      <c r="N75" s="6" t="inlineStr">
+      <c r="P75" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6003,17 +6459,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L76" s="6" t="inlineStr">
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M76" s="5" t="inlineStr"/>
+      <c r="N76" s="6" t="inlineStr">
         <is>
           <t>Simulasi delay</t>
         </is>
       </c>
-      <c r="M76" s="6" t="inlineStr">
+      <c r="O76" s="6" t="inlineStr">
         <is>
           <t>Skeleton saat data dimuat, bukan spinner kosong</t>
         </is>
       </c>
-      <c r="N76" s="6" t="inlineStr">
+      <c r="P76" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6075,17 +6537,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L77" s="4" t="inlineStr">
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="4" t="inlineStr">
         <is>
           <t>Posting jurnal 10jt → kembali ke Dashboard</t>
         </is>
       </c>
-      <c r="M77" s="4" t="inlineStr">
+      <c r="O77" s="4" t="inlineStr">
         <is>
           <t>Aset 557→567jt; Laba Bruto 44→54jt</t>
         </is>
       </c>
-      <c r="N77" s="4" t="inlineStr">
+      <c r="P77" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6147,17 +6615,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L78" s="4" t="inlineStr">
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="4" t="inlineStr">
         <is>
           <t>Buka laporan, periode 2026-03</t>
         </is>
       </c>
-      <c r="M78" s="4" t="inlineStr">
+      <c r="O78" s="4" t="inlineStr">
         <is>
           <t>Header perusahaan+judul+periode; section PENDAPATAN (subtotal 155jt) &amp; BEBAN (111jt); LABA/RUGI BERSIH 44jt bold</t>
         </is>
       </c>
-      <c r="N78" s="4" t="inlineStr">
+      <c r="P78" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6219,17 +6693,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L79" s="4" t="inlineStr">
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr"/>
+      <c r="N79" s="4" t="inlineStr">
         <is>
           <t>Hitung ulang dari seed</t>
         </is>
       </c>
-      <c r="M79" s="4" t="inlineStr">
+      <c r="O79" s="4" t="inlineStr">
         <is>
           <t>155jt − 111jt = 44jt (unit test juga)</t>
         </is>
       </c>
-      <c r="N79" s="4" t="inlineStr">
+      <c r="P79" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6291,17 +6771,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L80" s="6" t="inlineStr">
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M80" s="5" t="inlineStr"/>
+      <c r="N80" s="6" t="inlineStr">
         <is>
           <t>Periode tanpa transaksi</t>
         </is>
       </c>
-      <c r="M80" s="6" t="inlineStr">
+      <c r="O80" s="6" t="inlineStr">
         <is>
           <t>"Belum ada transaksi di periode ini" + link buat jurnal</t>
         </is>
       </c>
-      <c r="N80" s="6" t="inlineStr">
+      <c r="P80" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6363,17 +6849,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L81" s="6" t="inlineStr">
+      <c r="L81" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M81" s="5" t="inlineStr"/>
+      <c r="N81" s="6" t="inlineStr">
         <is>
           <t>Periksa baris laporan</t>
         </is>
       </c>
-      <c r="M81" s="6" t="inlineStr">
+      <c r="O81" s="6" t="inlineStr">
         <is>
           <t>Indentasi sesuai hierarki; format IDR konsisten</t>
         </is>
       </c>
-      <c r="N81" s="6" t="inlineStr">
+      <c r="P81" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6435,17 +6927,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L82" s="4" t="inlineStr">
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr"/>
+      <c r="N82" s="4" t="inlineStr">
         <is>
           <t>Buka Neraca, asOf 2026-03-31</t>
         </is>
       </c>
-      <c r="M82" s="4" t="inlineStr">
+      <c r="O82" s="4" t="inlineStr">
         <is>
           <t>"Per 31 Maret 2026"; section ASET &amp; KEWAJIBAN+EKUITAS; laba berjalan di ekuitas</t>
         </is>
       </c>
-      <c r="N82" s="4" t="inlineStr">
+      <c r="P82" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6507,17 +7005,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L83" s="4" t="inlineStr">
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr"/>
+      <c r="N83" s="4" t="inlineStr">
         <is>
           <t>Periksa indikator</t>
         </is>
       </c>
-      <c r="M83" s="4" t="inlineStr">
+      <c r="O83" s="4" t="inlineStr">
         <is>
           <t>Aset 557jt = Kewajiban+Ekuitas 557jt → ✓ hijau; jika dipecah saldo → ✗ merah + selisih</t>
         </is>
       </c>
-      <c r="N83" s="4" t="inlineStr">
+      <c r="P83" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6579,17 +7083,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L84" s="4" t="inlineStr">
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr"/>
+      <c r="N84" s="4" t="inlineStr">
         <is>
           <t>Jalankan test formula</t>
         </is>
       </c>
-      <c r="M84" s="4" t="inlineStr">
+      <c r="O84" s="4" t="inlineStr">
         <is>
           <t>balance_sheet seimbang dengan data mock</t>
         </is>
       </c>
-      <c r="N84" s="4" t="inlineStr">
+      <c r="P84" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6651,17 +7161,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L85" s="4" t="inlineStr">
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr"/>
+      <c r="N85" s="4" t="inlineStr">
         <is>
           <t>Buka trial balance Maret</t>
         </is>
       </c>
-      <c r="M85" s="4" t="inlineStr">
+      <c r="O85" s="4" t="inlineStr">
         <is>
           <t>Semua akun (kode, nama, debit, kredit); total debit = kredit = 668jt; ✓ indikator</t>
         </is>
       </c>
-      <c r="N85" s="4" t="inlineStr">
+      <c r="P85" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6723,17 +7239,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L86" s="6" t="inlineStr">
+      <c r="L86" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M86" s="5" t="inlineStr"/>
+      <c r="N86" s="6" t="inlineStr">
         <is>
           <t>Klik Kas Besar</t>
         </is>
       </c>
-      <c r="M86" s="6" t="inlineStr">
+      <c r="O86" s="6" t="inlineStr">
         <is>
           <t>Navigasi ke Buku Besar akun</t>
         </is>
       </c>
-      <c r="N86" s="6" t="inlineStr">
+      <c r="P86" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6795,17 +7317,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L87" s="6" t="inlineStr">
+      <c r="L87" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M87" s="5" t="inlineStr"/>
+      <c r="N87" s="6" t="inlineStr">
         <is>
           <t>Akun tanpa transaksi tapi ber-saldo awal</t>
         </is>
       </c>
-      <c r="M87" s="6" t="inlineStr">
+      <c r="O87" s="6" t="inlineStr">
         <is>
           <t>Muncul di neraca lajur</t>
         </is>
       </c>
-      <c r="N87" s="6" t="inlineStr">
+      <c r="P87" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6867,17 +7395,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L88" s="6" t="inlineStr">
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M88" s="5" t="inlineStr"/>
+      <c r="N88" s="6" t="inlineStr">
         <is>
           <t>Laba Rugi → "Bandingkan dengan: 2026-02"</t>
         </is>
       </c>
-      <c r="M88" s="6" t="inlineStr">
+      <c r="O88" s="6" t="inlineStr">
         <is>
           <t>Kolom/baris periode berjalan vs pembanding + selisih + delta % di total</t>
         </is>
       </c>
-      <c r="N88" s="6" t="inlineStr">
+      <c r="P88" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -6939,17 +7473,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L89" s="4" t="inlineStr">
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr"/>
+      <c r="N89" s="4" t="inlineStr">
         <is>
           <t>Export dari Laba Rugi Maret</t>
         </is>
       </c>
-      <c r="M89" s="4" t="inlineStr">
+      <c r="O89" s="4" t="inlineStr">
         <is>
           <t>File Laba-Rugi-Maret-2026.pdf; berisi kop, judul, periode, isi, footer; angka rata kanan IDR</t>
         </is>
       </c>
-      <c r="N89" s="4" t="inlineStr">
+      <c r="P89" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7011,17 +7551,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L90" s="6" t="inlineStr">
+      <c r="L90" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M90" s="5" t="inlineStr"/>
+      <c r="N90" s="6" t="inlineStr">
         <is>
           <t>Export Neraca per 31 Mar</t>
         </is>
       </c>
-      <c r="M90" s="6" t="inlineStr">
+      <c r="O90" s="6" t="inlineStr">
         <is>
           <t>Neraca-31-Maret-2026.pdf; isi benar</t>
         </is>
       </c>
-      <c r="N90" s="6" t="inlineStr">
+      <c r="P90" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7083,17 +7629,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L91" s="6" t="inlineStr">
+      <c r="L91" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M91" s="5" t="inlineStr"/>
+      <c r="N91" s="6" t="inlineStr">
         <is>
           <t>Export GL &amp; daftar jurnal</t>
         </is>
       </c>
-      <c r="M91" s="6" t="inlineStr">
+      <c r="O91" s="6" t="inlineStr">
         <is>
           <t>File terunduh, format rapi</t>
         </is>
       </c>
-      <c r="N91" s="6" t="inlineStr">
+      <c r="P91" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7155,17 +7707,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L92" s="6" t="inlineStr">
+      <c r="L92" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M92" s="5" t="inlineStr"/>
+      <c r="N92" s="6" t="inlineStr">
         <is>
           <t>Generate laporan besar</t>
         </is>
       </c>
-      <c r="M92" s="6" t="inlineStr">
+      <c r="O92" s="6" t="inlineStr">
         <is>
           <t>Progress bar saat generate (laporan tahunan)</t>
         </is>
       </c>
-      <c r="N92" s="6" t="inlineStr">
+      <c r="P92" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7227,17 +7785,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L93" s="6" t="inlineStr">
+      <c r="L93" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M93" s="5" t="inlineStr"/>
+      <c r="N93" s="6" t="inlineStr">
         <is>
           <t>Export Neraca Lajur → Excel</t>
         </is>
       </c>
-      <c r="M93" s="6" t="inlineStr">
+      <c r="O93" s="6" t="inlineStr">
         <is>
           <t>Neraca-Lajur-Maret-2026.xlsx; kolom rapi; nilai angka (bukan teks) agar bisa dihitung</t>
         </is>
       </c>
-      <c r="N93" s="6" t="inlineStr">
+      <c r="P93" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7299,17 +7863,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L94" s="4" t="inlineStr">
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="4" t="inlineStr">
         <is>
           <t>Bandingkan PDF/XLSX vs layar</t>
         </is>
       </c>
-      <c r="M94" s="4" t="inlineStr">
+      <c r="O94" s="4" t="inlineStr">
         <is>
           <t>Angka identik dengan laporan di layar</t>
         </is>
       </c>
-      <c r="N94" s="4" t="inlineStr">
+      <c r="P94" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7363,17 +7933,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L95" s="6" t="inlineStr">
+      <c r="L95" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M95" s="5" t="inlineStr"/>
+      <c r="N95" s="6" t="inlineStr">
         <is>
           <t>format=docx</t>
         </is>
       </c>
-      <c r="M95" s="6" t="inlineStr">
+      <c r="O95" s="6" t="inlineStr">
         <is>
           <t>422 UNSUPPORTED_FORMAT</t>
         </is>
       </c>
-      <c r="N95" s="6" t="inlineStr">
+      <c r="P95" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7435,17 +8011,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L96" s="4" t="inlineStr">
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr"/>
+      <c r="N96" s="4" t="inlineStr">
         <is>
           <t>Cek aksi di jurnal draft</t>
         </is>
       </c>
-      <c r="M96" s="4" t="inlineStr">
+      <c r="O96" s="4" t="inlineStr">
         <is>
           <t>Tombol Reverse hanya di jurnal posted; bukan hapus</t>
         </is>
       </c>
-      <c r="N96" s="4" t="inlineStr">
+      <c r="P96" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7507,17 +8089,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L97" s="4" t="inlineStr">
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="4" t="inlineStr">
         <is>
           <t>Reverse JNL-01 (Kas 25 / Pendapatan 25)</t>
         </is>
       </c>
-      <c r="M97" s="4" t="inlineStr">
+      <c r="O97" s="4" t="inlineStr">
         <is>
           <t>Dialog konfirmasi + pratinjau jurnal pembalik (D↔K); asal → reversed; pembalik auto-posted ref REV-BKM-2026-03-0001</t>
         </is>
       </c>
-      <c r="N97" s="4" t="inlineStr">
+      <c r="P97" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7579,17 +8167,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L98" s="4" t="inlineStr">
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="4" t="inlineStr">
         <is>
           <t>Setelah TC-RVS-02, cek saldo</t>
         </is>
       </c>
-      <c r="M98" s="4" t="inlineStr">
+      <c r="O98" s="4" t="inlineStr">
         <is>
           <t>Kas 87→62jt (25jt keluar); Pendapatan 155→130jt; pasangan asli+pembalik net 0</t>
         </is>
       </c>
-      <c r="N98" s="4" t="inlineStr">
+      <c r="P98" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7651,17 +8245,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L99" s="6" t="inlineStr">
+      <c r="L99" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M99" s="5" t="inlineStr"/>
+      <c r="N99" s="6" t="inlineStr">
         <is>
           <t>Reverse jurnal yang sudah reversed</t>
         </is>
       </c>
-      <c r="M99" s="6" t="inlineStr">
+      <c r="O99" s="6" t="inlineStr">
         <is>
           <t>409 ALREADY_REVERSED; tombol non-aktif</t>
         </is>
       </c>
-      <c r="N99" s="6" t="inlineStr">
+      <c r="P99" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7723,17 +8323,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L100" s="6" t="inlineStr">
+      <c r="L100" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M100" s="5" t="inlineStr"/>
+      <c r="N100" s="6" t="inlineStr">
         <is>
           <t>Periksa audit trail jurnal asal</t>
         </is>
       </c>
-      <c r="M100" s="6" t="inlineStr">
+      <c r="O100" s="6" t="inlineStr">
         <is>
           <t>Entry reverse (user, timestamp) tercatat</t>
         </is>
       </c>
-      <c r="N100" s="6" t="inlineStr">
+      <c r="P100" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7795,17 +8401,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L101" s="4" t="inlineStr">
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr"/>
+      <c r="N101" s="4" t="inlineStr">
         <is>
           <t>Upload dari form jurnal (drag-drop &amp; klik)</t>
         </is>
       </c>
-      <c r="M101" s="4" t="inlineStr">
+      <c r="O101" s="4" t="inlineStr">
         <is>
           <t>jpg/png/pdf diterima; maks 5MB &amp; 5 file; thumbnail/ikon di detail; bisa diunduh</t>
         </is>
       </c>
-      <c r="N101" s="4" t="inlineStr">
+      <c r="P101" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7867,17 +8479,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L102" s="6" t="inlineStr">
+      <c r="L102" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M102" s="5" t="inlineStr"/>
+      <c r="N102" s="6" t="inlineStr">
         <is>
           <t>Upload 6MB</t>
         </is>
       </c>
-      <c r="M102" s="6" t="inlineStr">
+      <c r="O102" s="6" t="inlineStr">
         <is>
           <t>Error "Ukuran file maksimal 5 MB" (422 FILE_TOO_LARGE)</t>
         </is>
       </c>
-      <c r="N102" s="6" t="inlineStr">
+      <c r="P102" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -7939,17 +8557,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L103" s="6" t="inlineStr">
+      <c r="L103" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M103" s="5" t="inlineStr"/>
+      <c r="N103" s="6" t="inlineStr">
         <is>
           <t>Upload .exe/.zip</t>
         </is>
       </c>
-      <c r="M103" s="6" t="inlineStr">
+      <c r="O103" s="6" t="inlineStr">
         <is>
           <t>Error "Tipe file tidak didukung" (422 UNSUPPORTED_FILE_TYPE)</t>
         </is>
       </c>
-      <c r="N103" s="6" t="inlineStr">
+      <c r="P103" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8011,17 +8635,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L104" s="6" t="inlineStr">
+      <c r="L104" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M104" s="5" t="inlineStr"/>
+      <c r="N104" s="6" t="inlineStr">
         <is>
           <t>Coba hapus lampiran jurnal posted</t>
         </is>
       </c>
-      <c r="M104" s="6" t="inlineStr">
+      <c r="O104" s="6" t="inlineStr">
         <is>
           <t>Diblokir 409 JOURNAL_ALREADY_POSTED (hanya sebelum posted)</t>
         </is>
       </c>
-      <c r="N104" s="6" t="inlineStr">
+      <c r="P104" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8083,17 +8713,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L105" s="4" t="inlineStr">
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr"/>
+      <c r="N105" s="4" t="inlineStr">
         <is>
           <t>Submit JNL-07</t>
         </is>
       </c>
-      <c r="M105" s="4" t="inlineStr">
+      <c r="O105" s="4" t="inlineStr">
         <is>
           <t>Status pending-approval; muncul di daftar &amp; alert dashboard</t>
         </is>
       </c>
-      <c r="N105" s="4" t="inlineStr">
+      <c r="P105" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8155,17 +8791,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L106" s="4" t="inlineStr">
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr"/>
+      <c r="N106" s="4" t="inlineStr">
         <is>
           <t>Approve sebagai admin (Rina)</t>
         </is>
       </c>
-      <c r="M106" s="4" t="inlineStr">
+      <c r="O106" s="4" t="inlineStr">
         <is>
           <t>Status posted; saldo ter-update; approvedBy/approvedAt terisi</t>
         </is>
       </c>
-      <c r="N106" s="4" t="inlineStr">
+      <c r="P106" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8227,17 +8869,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L107" s="6" t="inlineStr">
+      <c r="L107" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M107" s="5" t="inlineStr"/>
+      <c r="N107" s="6" t="inlineStr">
         <is>
           <t>Reject dengan alasan</t>
         </is>
       </c>
-      <c r="M107" s="6" t="inlineStr">
+      <c r="O107" s="6" t="inlineStr">
         <is>
           <t>Kembali draft; alasan wajib (kosong → ditolak); rejectionReason tersimpan</t>
         </is>
       </c>
-      <c r="N107" s="6" t="inlineStr">
+      <c r="P107" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8299,17 +8947,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L108" s="4" t="inlineStr">
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr"/>
+      <c r="N108" s="4" t="inlineStr">
         <is>
           <t>Login sebagai Dimas (accountant, tanpa approve)</t>
         </is>
       </c>
-      <c r="M108" s="4" t="inlineStr">
+      <c r="O108" s="4" t="inlineStr">
         <is>
           <t>Tombol approve tidak muncul (403 NO_APPROVAL_RIGHTS jika dipaksa)</t>
         </is>
       </c>
-      <c r="N108" s="4" t="inlineStr">
+      <c r="P108" s="4" t="inlineStr">
         <is>
           <t>Login sebagai Dimas (accountant) — tanpa izin approve</t>
         </is>
@@ -8371,17 +9025,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L109" s="6" t="inlineStr">
+      <c r="L109" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M109" s="5" t="inlineStr"/>
+      <c r="N109" s="6" t="inlineStr">
         <is>
           <t>Periksa dashboard</t>
         </is>
       </c>
-      <c r="M109" s="6" t="inlineStr">
+      <c r="O109" s="6" t="inlineStr">
         <is>
           <t>Notifikasi/badge jurnal menunggu approval</t>
         </is>
       </c>
-      <c r="N109" s="6" t="inlineStr">
+      <c r="P109" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8443,17 +9103,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L110" s="6" t="inlineStr">
+      <c r="L110" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M110" s="5" t="inlineStr"/>
+      <c r="N110" s="6" t="inlineStr">
         <is>
           <t>Approve jurnal draft (belum submit)</t>
         </is>
       </c>
-      <c r="M110" s="6" t="inlineStr">
+      <c r="O110" s="6" t="inlineStr">
         <is>
           <t>409 INVALID_STATUS_TRANSITION</t>
         </is>
       </c>
-      <c r="N110" s="6" t="inlineStr">
+      <c r="P110" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8515,17 +9181,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L111" s="4" t="inlineStr">
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M111" s="2" t="inlineStr"/>
+      <c r="N111" s="4" t="inlineStr">
         <is>
           <t>Admin → Pengaturan → Pengguna</t>
         </is>
       </c>
-      <c r="M111" s="4" t="inlineStr">
+      <c r="O111" s="4" t="inlineStr">
         <is>
           <t>Tambah/ubah/non-aktifkan user + assign role; 409 EMAIL_EXISTS untuk duplikat</t>
         </is>
       </c>
-      <c r="N111" s="4" t="inlineStr">
+      <c r="P111" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -8587,17 +9259,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L112" s="4" t="inlineStr">
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr"/>
+      <c r="N112" s="4" t="inlineStr">
         <is>
           <t>Login Budi (viewer)</t>
         </is>
       </c>
-      <c r="M112" s="4" t="inlineStr">
+      <c r="O112" s="4" t="inlineStr">
         <is>
           <t>Semua aksi tulis disabled (buat/edit/hapus jurnal); hanya baca</t>
         </is>
       </c>
-      <c r="N112" s="4" t="inlineStr">
+      <c r="P112" s="4" t="inlineStr">
         <is>
           <t>Login sebagai Budi (viewer)</t>
         </is>
@@ -8659,17 +9337,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L113" s="6" t="inlineStr">
+      <c r="L113" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M113" s="5" t="inlineStr"/>
+      <c r="N113" s="6" t="inlineStr">
         <is>
           <t>Login Dimas</t>
         </is>
       </c>
-      <c r="M113" s="6" t="inlineStr">
+      <c r="O113" s="6" t="inlineStr">
         <is>
           <t>Bisa entri jurnal, tidak bisa kelola user (403)</t>
         </is>
       </c>
-      <c r="N113" s="6" t="inlineStr">
+      <c r="P113" s="6" t="inlineStr">
         <is>
           <t>Login sebagai Dimas (accountant)</t>
         </is>
@@ -8731,17 +9415,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L114" s="6" t="inlineStr">
+      <c r="L114" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M114" s="5" t="inlineStr"/>
+      <c r="N114" s="6" t="inlineStr">
         <is>
           <t>Cek GET /auth/me tiap role</t>
         </is>
       </c>
-      <c r="M114" s="6" t="inlineStr">
+      <c r="O114" s="6" t="inlineStr">
         <is>
           <t>permissions sesuai role: admin 8 izin, accountant 4, viewer 2</t>
         </is>
       </c>
-      <c r="N114" s="6" t="inlineStr">
+      <c r="P114" s="6" t="inlineStr">
         <is>
           <t>Login bergantian sebagai Rina/Dimas/Budi</t>
         </is>
@@ -8803,17 +9493,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L115" s="4" t="inlineStr">
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr"/>
+      <c r="N115" s="4" t="inlineStr">
         <is>
           <t>Akuntan → dropdown entitas → CV Karya Mandiri</t>
         </is>
       </c>
-      <c r="M115" s="4" t="inlineStr">
+      <c r="O115" s="4" t="inlineStr">
         <is>
           <t>Seluruh data berganti (COA, jurnal, laporan); header laporan menampilkan nama entitas aktif</t>
         </is>
       </c>
-      <c r="N115" s="4" t="inlineStr">
+      <c r="P115" s="4" t="inlineStr">
         <is>
           <t>Login sebagai akuntan; entitas CV Karya Mandiri (ent-002) tersedia</t>
         </is>
@@ -8875,17 +9571,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L116" s="4" t="inlineStr">
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr"/>
+      <c r="N116" s="4" t="inlineStr">
         <is>
           <t>Di ent-002, cari jurnal ent-001</t>
         </is>
       </c>
-      <c r="M116" s="4" t="inlineStr">
+      <c r="O116" s="4" t="inlineStr">
         <is>
           <t>Tidak ada data bocor antar klien (filter X-Entity-Id)</t>
         </is>
       </c>
-      <c r="N116" s="4" t="inlineStr">
+      <c r="P116" s="4" t="inlineStr">
         <is>
           <t>Login sebagai akuntan; data ent-001 sudah terisi</t>
         </is>
@@ -8947,17 +9649,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L117" s="6" t="inlineStr">
+      <c r="L117" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M117" s="5" t="inlineStr"/>
+      <c r="N117" s="6" t="inlineStr">
         <is>
           <t>Pengaturan → Perusahaan</t>
         </is>
       </c>
-      <c r="M117" s="6" t="inlineStr">
+      <c r="O117" s="6" t="inlineStr">
         <is>
           <t>Ubah nama, mata uang (IDR), awal tahun fiskal</t>
         </is>
       </c>
-      <c r="N117" s="6" t="inlineStr">
+      <c r="P117" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9019,17 +9727,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L118" s="6" t="inlineStr">
+      <c r="L118" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M118" s="5" t="inlineStr"/>
+      <c r="N118" s="6" t="inlineStr">
         <is>
           <t>Buka tiap modul dengan delay</t>
         </is>
       </c>
-      <c r="M118" s="6" t="inlineStr">
+      <c r="O118" s="6" t="inlineStr">
         <is>
           <t>Skeleton/spinner di semua modul saat loading</t>
         </is>
       </c>
-      <c r="N118" s="6" t="inlineStr">
+      <c r="P118" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9091,17 +9805,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L119" s="4" t="inlineStr">
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M119" s="2" t="inlineStr"/>
+      <c r="N119" s="4" t="inlineStr">
         <is>
           <t>Matikan server → aksi</t>
         </is>
       </c>
-      <c r="M119" s="4" t="inlineStr">
+      <c r="O119" s="4" t="inlineStr">
         <is>
           <t>Error banner + tombol "Muat Ulang"; toast error server</t>
         </is>
       </c>
-      <c r="N119" s="4" t="inlineStr">
+      <c r="P119" s="4" t="inlineStr">
         <is>
           <t>Server mock API dimatikan</t>
         </is>
@@ -9163,17 +9883,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L120" s="4" t="inlineStr">
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr"/>
+      <c r="N120" s="4" t="inlineStr">
         <is>
           <t>Posting di periode tertutup</t>
         </is>
       </c>
-      <c r="M120" s="4" t="inlineStr">
+      <c r="O120" s="4" t="inlineStr">
         <is>
           <t>Blokir + pesan jelas (lihat TC-JRN-22)</t>
         </is>
       </c>
-      <c r="N120" s="4" t="inlineStr">
+      <c r="P120" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9235,17 +9961,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L121" s="6" t="inlineStr">
+      <c r="L121" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M121" s="5" t="inlineStr"/>
+      <c r="N121" s="6" t="inlineStr">
         <is>
           <t>Jurnal draft tidak balance</t>
         </is>
       </c>
-      <c r="M121" s="6" t="inlineStr">
+      <c r="O121" s="6" t="inlineStr">
         <is>
           <t>Alert dashboard "Terdapat jurnal draft tidak balance"</t>
         </is>
       </c>
-      <c r="N121" s="6" t="inlineStr">
+      <c r="P121" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9307,17 +10039,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L122" s="6" t="inlineStr">
+      <c r="L122" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M122" s="5" t="inlineStr"/>
+      <c r="N122" s="6" t="inlineStr">
         <is>
           <t>Pilih akun non-aktif di form</t>
         </is>
       </c>
-      <c r="M122" s="6" t="inlineStr">
+      <c r="O122" s="6" t="inlineStr">
         <is>
           <t>Tidak tersedia di dropdown</t>
         </is>
       </c>
-      <c r="N122" s="6" t="inlineStr">
+      <c r="P122" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9379,17 +10117,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L123" s="6" t="inlineStr">
+      <c r="L123" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M123" s="5" t="inlineStr"/>
+      <c r="N123" s="6" t="inlineStr">
         <is>
           <t>Tab/SHIFT+Tab di form jurnal</t>
         </is>
       </c>
-      <c r="M123" s="6" t="inlineStr">
+      <c r="O123" s="6" t="inlineStr">
         <is>
           <t>Fokus berpindah logis; focus ring terlihat</t>
         </is>
       </c>
-      <c r="N123" s="6" t="inlineStr">
+      <c r="P123" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9451,17 +10195,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L124" s="6" t="inlineStr">
+      <c r="L124" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M124" s="5" t="inlineStr"/>
+      <c r="N124" s="6" t="inlineStr">
         <is>
           <t>Inspeksi ikon &amp; tombol ikon</t>
         </is>
       </c>
-      <c r="M124" s="6" t="inlineStr">
+      <c r="O124" s="6" t="inlineStr">
         <is>
           <t>Label aria pada semua ikon; tooltip</t>
         </is>
       </c>
-      <c r="N124" s="6" t="inlineStr">
+      <c r="P124" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9523,17 +10273,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L125" s="6" t="inlineStr">
+      <c r="L125" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M125" s="5" t="inlineStr"/>
+      <c r="N125" s="6" t="inlineStr">
         <is>
           <t>Submit 2×</t>
         </is>
       </c>
-      <c r="M125" s="6" t="inlineStr">
+      <c r="O125" s="6" t="inlineStr">
         <is>
           <t>1 jurnal saja (lihat TC-JRN-25)</t>
         </is>
       </c>
-      <c r="N125" s="6" t="inlineStr">
+      <c r="P125" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9595,17 +10351,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L126" s="4" t="inlineStr">
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M126" s="2" t="inlineStr"/>
+      <c r="N126" s="4" t="inlineStr">
         <is>
           <t>Muat 10.000 baris jurnal</t>
         </is>
       </c>
-      <c r="M126" s="4" t="inlineStr">
+      <c r="O126" s="4" t="inlineStr">
         <is>
           <t>Tabel &amp; buku besar virtual-scroll; scroll halus tanpa jank</t>
         </is>
       </c>
-      <c r="N126" s="4" t="inlineStr">
+      <c r="P126" s="4" t="inlineStr">
         <is>
           <t>Seed 10.000 jurnal (POST /admin/seed-bulk)</t>
         </is>
@@ -9667,17 +10429,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L127" s="4" t="inlineStr">
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M127" s="2" t="inlineStr"/>
+      <c r="N127" s="4" t="inlineStr">
         <is>
           <t>Ukur dengan profiler</t>
         </is>
       </c>
-      <c r="M127" s="4" t="inlineStr">
+      <c r="O127" s="4" t="inlineStr">
         <is>
           <t>Render 10.000 baris &lt; 2 detik</t>
         </is>
       </c>
-      <c r="N127" s="4" t="inlineStr">
+      <c r="P127" s="4" t="inlineStr">
         <is>
           <t>Seed 10.000 jurnal (POST /admin/seed-bulk)</t>
         </is>
@@ -9739,17 +10507,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L128" s="6" t="inlineStr">
+      <c r="L128" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M128" s="5" t="inlineStr"/>
+      <c r="N128" s="6" t="inlineStr">
         <is>
           <t>Filter di data besar</t>
         </is>
       </c>
-      <c r="M128" s="6" t="inlineStr">
+      <c r="O128" s="6" t="inlineStr">
         <is>
           <t>Tetap responsif (tidak freeze)</t>
         </is>
       </c>
-      <c r="N128" s="6" t="inlineStr">
+      <c r="P128" s="6" t="inlineStr">
         <is>
           <t>Seed 10.000 jurnal (POST /admin/seed-bulk)</t>
         </is>
@@ -9811,17 +10585,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L129" s="6" t="inlineStr">
+      <c r="L129" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M129" s="5" t="inlineStr"/>
+      <c r="N129" s="6" t="inlineStr">
         <is>
           <t>Ukur bundle produksi</t>
         </is>
       </c>
-      <c r="M129" s="6" t="inlineStr">
+      <c r="O129" s="6" t="inlineStr">
         <is>
           <t>Awal &lt; 200KB gzip (code splitting per modul)</t>
         </is>
       </c>
-      <c r="N129" s="6" t="inlineStr">
+      <c r="P129" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9883,17 +10663,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L130" s="4" t="inlineStr">
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr"/>
+      <c r="N130" s="4" t="inlineStr">
         <is>
           <t>User baru masuk</t>
         </is>
       </c>
-      <c r="M130" s="4" t="inlineStr">
+      <c r="O130" s="4" t="inlineStr">
         <is>
           <t>Checklist: buat entitas → muat template COA → jurnal pertama; tooltip/spotlight elemen kunci; tombol "Lewati"</t>
         </is>
       </c>
-      <c r="N130" s="4" t="inlineStr">
+      <c r="P130" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -9955,17 +10741,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L131" s="6" t="inlineStr">
+      <c r="L131" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M131" s="5" t="inlineStr"/>
+      <c r="N131" s="6" t="inlineStr">
         <is>
           <t>Posting jurnal pertama</t>
         </is>
       </c>
-      <c r="M131" s="6" t="inlineStr">
+      <c r="O131" s="6" t="inlineStr">
         <is>
           <t>Onboarding dianggap selesai; progress tersimpan</t>
         </is>
       </c>
-      <c r="N131" s="6" t="inlineStr">
+      <c r="P131" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -10027,17 +10819,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L132" s="6" t="inlineStr">
+      <c r="L132" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M132" s="5" t="inlineStr"/>
+      <c r="N132" s="6" t="inlineStr">
         <is>
           <t>Ukur dari first login</t>
         </is>
       </c>
-      <c r="M132" s="6" t="inlineStr">
+      <c r="O132" s="6" t="inlineStr">
         <is>
           <t>&lt; 5 menit (target BRD)</t>
         </is>
       </c>
-      <c r="N132" s="6" t="inlineStr">
+      <c r="P132" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -10099,17 +10897,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L133" s="6" t="inlineStr">
+      <c r="L133" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M133" s="5" t="inlineStr"/>
+      <c r="N133" s="6" t="inlineStr">
         <is>
           <t>Cek menu integrasi bank tanpa partner</t>
         </is>
       </c>
-      <c r="M133" s="6" t="inlineStr">
+      <c r="O133" s="6" t="inlineStr">
         <is>
           <t>Fitur nonaktif (feature flag) dengan pesan jelas</t>
         </is>
       </c>
-      <c r="N133" s="6" t="inlineStr">
+      <c r="P133" s="6" t="inlineStr">
         <is>
           <t>Integrasi bank nonaktif (feature flag OFF)</t>
         </is>
@@ -10171,17 +10975,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L134" s="4" t="inlineStr">
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr"/>
+      <c r="N134" s="4" t="inlineStr">
         <is>
           <t>Sambungkan akun bank</t>
         </is>
       </c>
-      <c r="M134" s="4" t="inlineStr">
+      <c r="O134" s="4" t="inlineStr">
         <is>
           <t>Transaksi muncul sebagai jurnal draft siap posting</t>
         </is>
       </c>
-      <c r="N134" s="4" t="inlineStr">
+      <c r="P134" s="4" t="inlineStr">
         <is>
           <t>Integrasi bank aktif (partner terhubung)</t>
         </is>
@@ -10243,17 +11053,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L135" s="6" t="inlineStr">
+      <c r="L135" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M135" s="5" t="inlineStr"/>
+      <c r="N135" s="6" t="inlineStr">
         <is>
           <t>Transaksi bank vs jurnal existing</t>
         </is>
       </c>
-      <c r="M135" s="6" t="inlineStr">
+      <c r="O135" s="6" t="inlineStr">
         <is>
           <t>Match by nominal/tanggal; yang cocok ditandai</t>
         </is>
       </c>
-      <c r="N135" s="6" t="inlineStr">
+      <c r="P135" s="6" t="inlineStr">
         <is>
           <t>Integrasi bank aktif; ada jurnal existing untuk rekonsiliasi</t>
         </is>
@@ -10303,17 +11119,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L136" s="6" t="inlineStr">
+      <c r="L136" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M136" s="5" t="inlineStr"/>
+      <c r="N136" s="6" t="inlineStr">
         <is>
           <t>Login → buat jurnal 10jt → draft → posting → cek saldo COA &amp; dashboard → edit draft lain → hapus draft</t>
         </is>
       </c>
-      <c r="M136" s="6" t="inlineStr">
+      <c r="O136" s="6" t="inlineStr">
         <is>
           <t>Saldo Kas 87→97jt; draft tidak mengubah saldo; hapus draft tidak mengubah saldo</t>
         </is>
       </c>
-      <c r="N136" s="6" t="inlineStr">
+      <c r="P136" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10363,17 +11185,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L137" s="6" t="inlineStr">
+      <c r="L137" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M137" s="5" t="inlineStr"/>
+      <c r="N137" s="6" t="inlineStr">
         <is>
           <t>Posting jurnal → reverse → cek saldo &amp; laporan</t>
         </is>
       </c>
-      <c r="M137" s="6" t="inlineStr">
+      <c r="O137" s="6" t="inlineStr">
         <is>
           <t>Kas kembali ke kondisi sebelum posting; trial balance tetap seimbang; jurnal asal reversed + pembalik posted</t>
         </is>
       </c>
-      <c r="N137" s="6" t="inlineStr">
+      <c r="P137" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10423,17 +11251,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L138" s="6" t="inlineStr">
+      <c r="L138" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M138" s="5" t="inlineStr"/>
+      <c r="N138" s="6" t="inlineStr">
         <is>
           <t>Posting jurnal baru → buka Laba Rugi/Neraca/Neraca Lajur → export PDF &amp; XLSX</t>
         </is>
       </c>
-      <c r="M138" s="6" t="inlineStr">
+      <c r="O138" s="6" t="inlineStr">
         <is>
           <t>Angka laporan &amp; export konsisten dengan saldo baru; neraca seimbang</t>
         </is>
       </c>
-      <c r="N138" s="6" t="inlineStr">
+      <c r="P138" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10483,17 +11317,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L139" s="6" t="inlineStr">
+      <c r="L139" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M139" s="5" t="inlineStr"/>
+      <c r="N139" s="6" t="inlineStr">
         <is>
           <t>Tutup Maret (post-all draft) → coba entri/posting → buka laporan</t>
         </is>
       </c>
-      <c r="M139" s="6" t="inlineStr">
+      <c r="O139" s="6" t="inlineStr">
         <is>
           <t>Entri/posting diblokir; laporan tetap bisa dibaca; draft ter-post via post-all muncul di laporan</t>
         </is>
       </c>
-      <c r="N139" s="6" t="inlineStr">
+      <c r="P139" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10543,17 +11383,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L140" s="6" t="inlineStr">
+      <c r="L140" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M140" s="5" t="inlineStr"/>
+      <c r="N140" s="6" t="inlineStr">
         <is>
           <t>Switch ke ent-002 → buat jurnal → switch balik ke ent-001</t>
         </is>
       </c>
-      <c r="M140" s="6" t="inlineStr">
+      <c r="O140" s="6" t="inlineStr">
         <is>
           <t>Data terisolasi; tidak ada silang; header entitas benar</t>
         </is>
       </c>
-      <c r="N140" s="6" t="inlineStr">
+      <c r="P140" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10603,17 +11449,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L141" s="6" t="inlineStr">
+      <c r="L141" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M141" s="5" t="inlineStr"/>
+      <c r="N141" s="6" t="inlineStr">
         <is>
           <t>Submit → approve (saldo berubah) → submit → reject (kembali draft, saldo tidak berubah)</t>
         </is>
       </c>
-      <c r="M141" s="6" t="inlineStr">
+      <c r="O141" s="6" t="inlineStr">
         <is>
           <t>Saldo hanya berubah saat approve; audit trail lengkap</t>
         </is>
       </c>
-      <c r="N141" s="6" t="inlineStr">
+      <c r="P141" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10663,17 +11515,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L142" s="6" t="inlineStr">
+      <c r="L142" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M142" s="5" t="inlineStr"/>
+      <c r="N142" s="6" t="inlineStr">
         <is>
           <t>Filter jurnal → search global → klik hasil → buka detail</t>
         </is>
       </c>
-      <c r="M142" s="6" t="inlineStr">
+      <c r="O142" s="6" t="inlineStr">
         <is>
           <t>Navigasi benar; filter tersimpan di URL; keyword konsisten</t>
         </is>
       </c>
-      <c r="N142" s="6" t="inlineStr">
+      <c r="P142" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10723,17 +11581,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L143" s="6" t="inlineStr">
+      <c r="L143" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M143" s="5" t="inlineStr"/>
+      <c r="N143" s="6" t="inlineStr">
         <is>
           <t>Ganti periode → semua laporan re-fetch</t>
         </is>
       </c>
-      <c r="M143" s="6" t="inlineStr">
+      <c r="O143" s="6" t="inlineStr">
         <is>
           <t>Dashboard, Laba Rugi, Neraca, Buku Besar, Neraca Lajur sinkron</t>
         </is>
       </c>
-      <c r="N143" s="6" t="inlineStr">
+      <c r="P143" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10783,17 +11647,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L144" s="6" t="inlineStr">
+      <c r="L144" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M144" s="5" t="inlineStr"/>
+      <c r="N144" s="6" t="inlineStr">
         <is>
           <t>Muat 10.000 jurnal → scroll, filter, export</t>
         </is>
       </c>
-      <c r="M144" s="6" t="inlineStr">
+      <c r="O144" s="6" t="inlineStr">
         <is>
           <t>&lt; 2 detik render, tanpa jank, angka tetap benar</t>
         </is>
       </c>
-      <c r="N144" s="6" t="inlineStr">
+      <c r="P144" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10843,17 +11713,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L145" s="6" t="inlineStr">
+      <c r="L145" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M145" s="5" t="inlineStr"/>
+      <c r="N145" s="6" t="inlineStr">
         <is>
           <t>Posting jurnal → restart server</t>
         </is>
       </c>
-      <c r="M145" s="6" t="inlineStr">
+      <c r="O145" s="6" t="inlineStr">
         <is>
           <t>Data kembali ke seed (in-memory) — dokumentasikan; tidak ada error UI setelah restart</t>
         </is>
       </c>
-      <c r="N145" s="6" t="inlineStr">
+      <c r="P145" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10903,17 +11779,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L146" s="6" t="inlineStr">
+      <c r="L146" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M146" s="5" t="inlineStr"/>
+      <c r="N146" s="6" t="inlineStr">
         <is>
           <t>Jalankan suite E2E di Chrome + Firefox</t>
         </is>
       </c>
-      <c r="M146" s="6" t="inlineStr">
+      <c r="O146" s="6" t="inlineStr">
         <is>
           <t>Tidak ada perbedaan perilaku; layout mobile 320px OK</t>
         </is>
       </c>
-      <c r="N146" s="6" t="inlineStr">
+      <c r="P146" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -10963,17 +11845,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L147" s="6" t="inlineStr">
+      <c r="L147" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M147" s="5" t="inlineStr"/>
+      <c r="N147" s="6" t="inlineStr">
         <is>
           <t>Server mati → semua modul</t>
         </is>
       </c>
-      <c r="M147" s="6" t="inlineStr">
+      <c r="O147" s="6" t="inlineStr">
         <is>
           <t>Banner error + "Muat Ulang"; tidak ada crash/halaman putih</t>
         </is>
       </c>
-      <c r="N147" s="6" t="inlineStr">
+      <c r="P147" s="6" t="inlineStr">
         <is>
           <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
@@ -11035,17 +11923,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L148" s="4" t="inlineStr">
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr"/>
+      <c r="N148" s="4" t="inlineStr">
         <is>
           <t>Buka laporan Arus Kas Maret</t>
         </is>
       </c>
-      <c r="M148" s="4" t="inlineStr">
+      <c r="O148" s="4" t="inlineStr">
         <is>
           <t>Seksi Operasi / Investasi / Pendanaan dengan subtotal; metode tidak langsung</t>
         </is>
       </c>
-      <c r="N148" s="4" t="inlineStr">
+      <c r="P148" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -11107,17 +12001,23 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L149" s="4" t="inlineStr">
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr"/>
+      <c r="N149" s="4" t="inlineStr">
         <is>
           <t>Cek formula</t>
         </is>
       </c>
-      <c r="M149" s="4" t="inlineStr">
+      <c r="O149" s="4" t="inlineStr">
         <is>
           <t>Kas akhir = kas awal + arus kas bersih (unit test)</t>
         </is>
       </c>
-      <c r="N149" s="4" t="inlineStr">
+      <c r="P149" s="4" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
@@ -11179,24 +12079,30 @@
           <t>QA Local (mock API)</t>
         </is>
       </c>
-      <c r="L150" s="6" t="inlineStr">
+      <c r="L150" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M150" s="5" t="inlineStr"/>
+      <c r="N150" s="6" t="inlineStr">
         <is>
           <t>Ubah mapping di Pengaturan</t>
         </is>
       </c>
-      <c r="M150" s="6" t="inlineStr">
+      <c r="O150" s="6" t="inlineStr">
         <is>
           <t>Perubahan mapping tercermin di laporan</t>
         </is>
       </c>
-      <c r="N150" s="6" t="inlineStr">
+      <c r="P150" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N150"/>
+  <autoFilter ref="A1:P150"/>
   <conditionalFormatting sqref="I2:I150">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>$I2="Passed"</formula>

</xml_diff>

<commit_message>
feat(qa): conditional formatting Status di daftar S1 sheet Ringkasan — konsisten dengan Test Cases
- write_xlsx: kolom Status di bagian "Peringatan S1 (Not Run/Fail)" kini memakai
  add_status_cf yang sama dengan sheet Test Cases (Passed hijau, Fail/Failed
  merah, Not Run abu-abu, Blocked/Retest amber, Skipped biru-abu) — range
  B<first>:B<last> di daftar S1 yang belum lolos
- qa-test-cases.xlsx diregenerasi: Ringkasan kini punya 1 CF range (B43:B96)
  selain Test Cases (I2:I150)
- Verifikasi: gate check-qa-sync [OK], 149 test case, tanggal run 2026-08-16
</commit_message>
<xml_diff>
--- a/qa-test-cases.xlsx
+++ b/qa-test-cases.xlsx
@@ -13188,6 +13188,23 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B43:B96">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>$B43="Passed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="0">
+      <formula>$B43="Fail" OR $B43="Failed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="0">
+      <formula>$B43="Not Run"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="0">
+      <formula>$B43="Blocked" OR $B43="Retest"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="0">
+      <formula>$B43="Skipped"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(qa): skenario RG-20/21/22 di QA Test Plan + CHANGELOG & README --only
RG-20 (SESSION_EXPIRED), RG-21/22 (RATE_LIMITED retry pulih/diblokir) jadi
skenario resmi §4 (EXPECTED_RG 13→15), artefak QA diregenerasi (137 TC + 15
RG = 152). CHANGELOG: modal Sesi Berakhir, NO_APPROVAL_RIGHTS, RG-20b/06e,
opsi --only. README: dokumentasi npm test -- --only=mock-api|prototype|e2e.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/qa-test-cases.xlsx
+++ b/qa-test-cases.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$P$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$P$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P150"/>
+  <dimension ref="A1:P153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11868,202 +11868,166 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t>TC-CFL-01</t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
-        <is>
-          <t>Arus Kas</t>
-        </is>
-      </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>3 seksi arus kas</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
-        <is>
-          <t>1 - Critical</t>
-        </is>
-      </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="G148" s="2" t="inlineStr">
-        <is>
-          <t>AAJ-028</t>
-        </is>
-      </c>
-      <c r="H148" s="2" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
-      <c r="I148" s="3" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J148" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="K148" s="2" t="inlineStr">
-        <is>
-          <t>QA Local (mock API)</t>
-        </is>
-      </c>
-      <c r="L148" s="2" t="inlineStr">
-        <is>
-          <t>Tim QA</t>
-        </is>
-      </c>
-      <c r="M148" s="2" t="inlineStr"/>
-      <c r="N148" s="4" t="inlineStr">
-        <is>
-          <t>Buka laporan Arus Kas Maret</t>
-        </is>
-      </c>
-      <c r="O148" s="4" t="inlineStr">
-        <is>
-          <t>Seksi Operasi / Investasi / Pendanaan dengan subtotal; metode tidak langsung</t>
-        </is>
-      </c>
-      <c r="P148" s="4" t="inlineStr">
-        <is>
-          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>RG-20</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>Skenario Regresi</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>SESSION_EXPIRED — refresh token kedaluwarsa di server</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>3 - Medium</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr"/>
+      <c r="G148" s="5" t="inlineStr"/>
+      <c r="H148" s="5" t="inlineStr"/>
+      <c r="I148" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="J148" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="K148" s="5" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L148" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M148" s="5" t="inlineStr"/>
+      <c r="N148" s="6" t="inlineStr">
+        <is>
+          <t>Login → POST /admin/expire-refresh-tokens (semua refresh token basi) + akses token dipaksa basi → pemicu fetch/reload → auto-refresh gagal 401 SESSION_EXPIRED → modal "Sesi Berakhir" → "Masuk kembali" → login ulang</t>
+        </is>
+      </c>
+      <c r="O148" s="6" t="inlineStr">
+        <is>
+          <t>Modal "Sesi Berakhir" muncul (bukan sekadar error inline); logout otomatis — token dibersihkan dari localStorage; login ulang wajib → sesi baru dengan token baru</t>
+        </is>
+      </c>
+      <c r="P148" s="6" t="inlineStr">
+        <is>
+          <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>TC-CFL-02</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
-        <is>
-          <t>Arus Kas</t>
-        </is>
-      </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>Konsistensi kas</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="E149" s="2" t="inlineStr">
-        <is>
-          <t>1 - Critical</t>
-        </is>
-      </c>
-      <c r="F149" s="2" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="G149" s="2" t="inlineStr">
-        <is>
-          <t>AAJ-028</t>
-        </is>
-      </c>
-      <c r="H149" s="2" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
-      <c r="I149" s="3" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J149" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="K149" s="2" t="inlineStr">
-        <is>
-          <t>QA Local (mock API)</t>
-        </is>
-      </c>
-      <c r="L149" s="2" t="inlineStr">
-        <is>
-          <t>Tim QA</t>
-        </is>
-      </c>
-      <c r="M149" s="2" t="inlineStr"/>
-      <c r="N149" s="4" t="inlineStr">
-        <is>
-          <t>Cek formula</t>
-        </is>
-      </c>
-      <c r="O149" s="4" t="inlineStr">
-        <is>
-          <t>Kas akhir = kas awal + arus kas bersih (unit test)</t>
-        </is>
-      </c>
-      <c r="P149" s="4" t="inlineStr">
-        <is>
-          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>RG-21</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Skenario Regresi</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>RATE_LIMITED — retry otomatis pulih</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>3 - Medium</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr"/>
+      <c r="G149" s="5" t="inlineStr"/>
+      <c r="H149" s="5" t="inlineStr"/>
+      <c r="I149" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="J149" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L149" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M149" s="5" t="inlineStr"/>
+      <c r="N149" s="6" t="inlineStr">
+        <is>
+          <t>POST /admin/set-rate-limit (ambang 1 req/endpoint) → simpan jurnal #1 (200) → simpan jurnal #2 kena 429 → klien retry otomatis (jeda Retry-After, cap 5 dtk) → ambang dinaikkan → retry berhasil</t>
+        </is>
+      </c>
+      <c r="O149" s="6" t="inlineStr">
+        <is>
+          <t>Jurnal #1 &amp; #2 tersimpan (8 seed + 2); TIDAK ada toast "Terlalu banyak permintaan"; bukti jaringan 429 → retry 201; sesi tetap aktif</t>
+        </is>
+      </c>
+      <c r="P149" s="6" t="inlineStr">
+        <is>
+          <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
         <is>
-          <t>TC-CFL-03</t>
+          <t>RG-22</t>
         </is>
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>Arus Kas</t>
+          <t>Skenario Regresi</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>Mapping grup akun</t>
+          <t>RATE_LIMITED — tetap diblokir</t>
         </is>
       </c>
       <c r="D150" s="5" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>2 - High</t>
-        </is>
-      </c>
-      <c r="F150" s="7" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="G150" s="5" t="inlineStr">
-        <is>
-          <t>AAJ-028</t>
-        </is>
-      </c>
-      <c r="H150" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
+          <t>3 - Medium</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr"/>
+      <c r="G150" s="5" t="inlineStr"/>
+      <c r="H150" s="5" t="inlineStr"/>
       <c r="I150" s="5" t="inlineStr">
         <is>
           <t>Not Run</t>
@@ -12087,23 +12051,257 @@
       <c r="M150" s="5" t="inlineStr"/>
       <c r="N150" s="6" t="inlineStr">
         <is>
+          <t>Ambang 1 + window panjang → simpan #1 (200) → simpan #2 kena 429 ×3 (1 asli + 2 retry, semua 429)</t>
+        </is>
+      </c>
+      <c r="O150" s="6" t="inlineStr">
+        <is>
+          <t>Toast "Terlalu banyak permintaan" tampil; jurnal #2 TIDAK tersimpan (daftar tetap 9 entri); sesi tetap aktif (429 ≠ logout)</t>
+        </is>
+      </c>
+      <c r="P150" s="6" t="inlineStr">
+        <is>
+          <t>State seed; mock API + prototipe berjalan (localhost:4000 / :5173)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>TC-CFL-01</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Arus Kas</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>3 seksi arus kas</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>1 - Critical</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>AAJ-028</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr"/>
+      <c r="N151" s="4" t="inlineStr">
+        <is>
+          <t>Buka laporan Arus Kas Maret</t>
+        </is>
+      </c>
+      <c r="O151" s="4" t="inlineStr">
+        <is>
+          <t>Seksi Operasi / Investasi / Pendanaan dengan subtotal; metode tidak langsung</t>
+        </is>
+      </c>
+      <c r="P151" s="4" t="inlineStr">
+        <is>
+          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>TC-CFL-02</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Arus Kas</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Konsistensi kas</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>1 - Critical</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>AAJ-028</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr"/>
+      <c r="N152" s="4" t="inlineStr">
+        <is>
+          <t>Cek formula</t>
+        </is>
+      </c>
+      <c r="O152" s="4" t="inlineStr">
+        <is>
+          <t>Kas akhir = kas awal + arus kas bersih (unit test)</t>
+        </is>
+      </c>
+      <c r="P152" s="4" t="inlineStr">
+        <is>
+          <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>TC-CFL-03</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Arus Kas</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>Mapping grup akun</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>2 - High</t>
+        </is>
+      </c>
+      <c r="F153" s="7" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>AAJ-028</t>
+        </is>
+      </c>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="I153" s="5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="J153" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="K153" s="5" t="inlineStr">
+        <is>
+          <t>QA Local (mock API)</t>
+        </is>
+      </c>
+      <c r="L153" s="5" t="inlineStr">
+        <is>
+          <t>Tim QA</t>
+        </is>
+      </c>
+      <c r="M153" s="5" t="inlineStr"/>
+      <c r="N153" s="6" t="inlineStr">
+        <is>
           <t>Ubah mapping di Pengaturan</t>
         </is>
       </c>
-      <c r="O150" s="6" t="inlineStr">
+      <c r="O153" s="6" t="inlineStr">
         <is>
           <t>Perubahan mapping tercermin di laporan</t>
         </is>
       </c>
-      <c r="P150" s="6" t="inlineStr">
+      <c r="P153" s="6" t="inlineStr">
         <is>
           <t>Reset data seed (mock API di-reset); login sebagai Rina (admin)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P150"/>
-  <conditionalFormatting sqref="I2:I150">
+  <autoFilter ref="A1:P153"/>
+  <conditionalFormatting sqref="I2:I153">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>$I2="Passed"</formula>
     </cfRule>
@@ -12156,7 +12354,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
@@ -12176,7 +12374,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5"/>

</xml_diff>